<commit_message>
Class groups: schema, grade helpers, categories API, server-side class lookups
A group is an ordinary top-level class; a grade is a sub-class (parentId)
and a child may carry an optional subCategoryId label (display, filter and
sort only, never access control). Adds src/lib/classGroups.ts (ordering,
tolerant grade matcher, validation), grades in GET/POST/PATCH/archive of
categories, grade validation on child create/update/import/approve, the
Grade import column and template, and parentId: null on every server-side
class lookup. Grades are archive-only; a group takes its grades to Trash
with it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XCzGEPT4UYsXTrWu42jKts
</commit_message>
<xml_diff>
--- a/public/templates/crechely-children-template.xlsx
+++ b/public/templates/crechely-children-template.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB500"/>
+  <dimension ref="A1:AC500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -504,6 +504,7 @@
     <col width="25" customWidth="1" min="26" max="26"/>
     <col width="28" customWidth="1" min="27" max="27"/>
     <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -647,6 +648,11 @@
           <t>Emergency Contact Phone</t>
         </is>
       </c>
+      <c r="AC1" s="4" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -769,6 +775,7 @@
           <t>084 000 0000</t>
         </is>
       </c>
+      <c r="AC2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="C3" s="7" t="n"/>
@@ -782,6 +789,7 @@
       <c r="V3" s="7" t="n"/>
       <c r="Y3" s="7" t="n"/>
       <c r="AB3" s="7" t="n"/>
+      <c r="AC3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="C4" s="7" t="n"/>
@@ -795,6 +803,7 @@
       <c r="V4" s="7" t="n"/>
       <c r="Y4" s="7" t="n"/>
       <c r="AB4" s="7" t="n"/>
+      <c r="AC4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="C5" s="7" t="n"/>
@@ -808,6 +817,7 @@
       <c r="V5" s="7" t="n"/>
       <c r="Y5" s="7" t="n"/>
       <c r="AB5" s="7" t="n"/>
+      <c r="AC5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="C6" s="7" t="n"/>
@@ -821,6 +831,7 @@
       <c r="V6" s="7" t="n"/>
       <c r="Y6" s="7" t="n"/>
       <c r="AB6" s="7" t="n"/>
+      <c r="AC6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="C7" s="7" t="n"/>
@@ -834,6 +845,7 @@
       <c r="V7" s="7" t="n"/>
       <c r="Y7" s="7" t="n"/>
       <c r="AB7" s="7" t="n"/>
+      <c r="AC7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="C8" s="7" t="n"/>
@@ -847,6 +859,7 @@
       <c r="V8" s="7" t="n"/>
       <c r="Y8" s="7" t="n"/>
       <c r="AB8" s="7" t="n"/>
+      <c r="AC8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="C9" s="7" t="n"/>
@@ -860,6 +873,7 @@
       <c r="V9" s="7" t="n"/>
       <c r="Y9" s="7" t="n"/>
       <c r="AB9" s="7" t="n"/>
+      <c r="AC9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="C10" s="7" t="n"/>
@@ -873,6 +887,7 @@
       <c r="V10" s="7" t="n"/>
       <c r="Y10" s="7" t="n"/>
       <c r="AB10" s="7" t="n"/>
+      <c r="AC10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="C11" s="7" t="n"/>
@@ -886,6 +901,7 @@
       <c r="V11" s="7" t="n"/>
       <c r="Y11" s="7" t="n"/>
       <c r="AB11" s="7" t="n"/>
+      <c r="AC11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="C12" s="7" t="n"/>
@@ -899,6 +915,7 @@
       <c r="V12" s="7" t="n"/>
       <c r="Y12" s="7" t="n"/>
       <c r="AB12" s="7" t="n"/>
+      <c r="AC12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="C13" s="7" t="n"/>
@@ -912,6 +929,7 @@
       <c r="V13" s="7" t="n"/>
       <c r="Y13" s="7" t="n"/>
       <c r="AB13" s="7" t="n"/>
+      <c r="AC13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="C14" s="7" t="n"/>
@@ -925,6 +943,7 @@
       <c r="V14" s="7" t="n"/>
       <c r="Y14" s="7" t="n"/>
       <c r="AB14" s="7" t="n"/>
+      <c r="AC14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="C15" s="7" t="n"/>
@@ -938,6 +957,7 @@
       <c r="V15" s="7" t="n"/>
       <c r="Y15" s="7" t="n"/>
       <c r="AB15" s="7" t="n"/>
+      <c r="AC15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="C16" s="7" t="n"/>
@@ -951,6 +971,7 @@
       <c r="V16" s="7" t="n"/>
       <c r="Y16" s="7" t="n"/>
       <c r="AB16" s="7" t="n"/>
+      <c r="AC16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="C17" s="7" t="n"/>
@@ -964,6 +985,7 @@
       <c r="V17" s="7" t="n"/>
       <c r="Y17" s="7" t="n"/>
       <c r="AB17" s="7" t="n"/>
+      <c r="AC17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="C18" s="7" t="n"/>
@@ -977,6 +999,7 @@
       <c r="V18" s="7" t="n"/>
       <c r="Y18" s="7" t="n"/>
       <c r="AB18" s="7" t="n"/>
+      <c r="AC18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="C19" s="7" t="n"/>
@@ -990,6 +1013,7 @@
       <c r="V19" s="7" t="n"/>
       <c r="Y19" s="7" t="n"/>
       <c r="AB19" s="7" t="n"/>
+      <c r="AC19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="C20" s="7" t="n"/>
@@ -1003,6 +1027,7 @@
       <c r="V20" s="7" t="n"/>
       <c r="Y20" s="7" t="n"/>
       <c r="AB20" s="7" t="n"/>
+      <c r="AC20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="C21" s="7" t="n"/>
@@ -1016,6 +1041,7 @@
       <c r="V21" s="7" t="n"/>
       <c r="Y21" s="7" t="n"/>
       <c r="AB21" s="7" t="n"/>
+      <c r="AC21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="C22" s="7" t="n"/>
@@ -1029,6 +1055,7 @@
       <c r="V22" s="7" t="n"/>
       <c r="Y22" s="7" t="n"/>
       <c r="AB22" s="7" t="n"/>
+      <c r="AC22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="C23" s="7" t="n"/>
@@ -1042,6 +1069,7 @@
       <c r="V23" s="7" t="n"/>
       <c r="Y23" s="7" t="n"/>
       <c r="AB23" s="7" t="n"/>
+      <c r="AC23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="C24" s="7" t="n"/>
@@ -1055,6 +1083,7 @@
       <c r="V24" s="7" t="n"/>
       <c r="Y24" s="7" t="n"/>
       <c r="AB24" s="7" t="n"/>
+      <c r="AC24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="C25" s="7" t="n"/>
@@ -1068,6 +1097,7 @@
       <c r="V25" s="7" t="n"/>
       <c r="Y25" s="7" t="n"/>
       <c r="AB25" s="7" t="n"/>
+      <c r="AC25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="C26" s="7" t="n"/>
@@ -1081,6 +1111,7 @@
       <c r="V26" s="7" t="n"/>
       <c r="Y26" s="7" t="n"/>
       <c r="AB26" s="7" t="n"/>
+      <c r="AC26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="C27" s="7" t="n"/>
@@ -1094,6 +1125,7 @@
       <c r="V27" s="7" t="n"/>
       <c r="Y27" s="7" t="n"/>
       <c r="AB27" s="7" t="n"/>
+      <c r="AC27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="C28" s="7" t="n"/>
@@ -1107,6 +1139,7 @@
       <c r="V28" s="7" t="n"/>
       <c r="Y28" s="7" t="n"/>
       <c r="AB28" s="7" t="n"/>
+      <c r="AC28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="C29" s="7" t="n"/>
@@ -1120,6 +1153,7 @@
       <c r="V29" s="7" t="n"/>
       <c r="Y29" s="7" t="n"/>
       <c r="AB29" s="7" t="n"/>
+      <c r="AC29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="C30" s="7" t="n"/>
@@ -1133,6 +1167,7 @@
       <c r="V30" s="7" t="n"/>
       <c r="Y30" s="7" t="n"/>
       <c r="AB30" s="7" t="n"/>
+      <c r="AC30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="C31" s="7" t="n"/>
@@ -1146,6 +1181,7 @@
       <c r="V31" s="7" t="n"/>
       <c r="Y31" s="7" t="n"/>
       <c r="AB31" s="7" t="n"/>
+      <c r="AC31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="C32" s="7" t="n"/>
@@ -1159,6 +1195,7 @@
       <c r="V32" s="7" t="n"/>
       <c r="Y32" s="7" t="n"/>
       <c r="AB32" s="7" t="n"/>
+      <c r="AC32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="C33" s="7" t="n"/>
@@ -1172,6 +1209,7 @@
       <c r="V33" s="7" t="n"/>
       <c r="Y33" s="7" t="n"/>
       <c r="AB33" s="7" t="n"/>
+      <c r="AC33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="C34" s="7" t="n"/>
@@ -1185,6 +1223,7 @@
       <c r="V34" s="7" t="n"/>
       <c r="Y34" s="7" t="n"/>
       <c r="AB34" s="7" t="n"/>
+      <c r="AC34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="C35" s="7" t="n"/>
@@ -1198,6 +1237,7 @@
       <c r="V35" s="7" t="n"/>
       <c r="Y35" s="7" t="n"/>
       <c r="AB35" s="7" t="n"/>
+      <c r="AC35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="C36" s="7" t="n"/>
@@ -1211,6 +1251,7 @@
       <c r="V36" s="7" t="n"/>
       <c r="Y36" s="7" t="n"/>
       <c r="AB36" s="7" t="n"/>
+      <c r="AC36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="C37" s="7" t="n"/>
@@ -1224,6 +1265,7 @@
       <c r="V37" s="7" t="n"/>
       <c r="Y37" s="7" t="n"/>
       <c r="AB37" s="7" t="n"/>
+      <c r="AC37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="C38" s="7" t="n"/>
@@ -1237,6 +1279,7 @@
       <c r="V38" s="7" t="n"/>
       <c r="Y38" s="7" t="n"/>
       <c r="AB38" s="7" t="n"/>
+      <c r="AC38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="C39" s="7" t="n"/>
@@ -1250,6 +1293,7 @@
       <c r="V39" s="7" t="n"/>
       <c r="Y39" s="7" t="n"/>
       <c r="AB39" s="7" t="n"/>
+      <c r="AC39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="C40" s="7" t="n"/>
@@ -1263,6 +1307,7 @@
       <c r="V40" s="7" t="n"/>
       <c r="Y40" s="7" t="n"/>
       <c r="AB40" s="7" t="n"/>
+      <c r="AC40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="C41" s="7" t="n"/>
@@ -1276,6 +1321,7 @@
       <c r="V41" s="7" t="n"/>
       <c r="Y41" s="7" t="n"/>
       <c r="AB41" s="7" t="n"/>
+      <c r="AC41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="C42" s="7" t="n"/>
@@ -1289,6 +1335,7 @@
       <c r="V42" s="7" t="n"/>
       <c r="Y42" s="7" t="n"/>
       <c r="AB42" s="7" t="n"/>
+      <c r="AC42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="C43" s="7" t="n"/>
@@ -1302,6 +1349,7 @@
       <c r="V43" s="7" t="n"/>
       <c r="Y43" s="7" t="n"/>
       <c r="AB43" s="7" t="n"/>
+      <c r="AC43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="C44" s="7" t="n"/>
@@ -1315,6 +1363,7 @@
       <c r="V44" s="7" t="n"/>
       <c r="Y44" s="7" t="n"/>
       <c r="AB44" s="7" t="n"/>
+      <c r="AC44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="C45" s="7" t="n"/>
@@ -1328,6 +1377,7 @@
       <c r="V45" s="7" t="n"/>
       <c r="Y45" s="7" t="n"/>
       <c r="AB45" s="7" t="n"/>
+      <c r="AC45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="C46" s="7" t="n"/>
@@ -1341,6 +1391,7 @@
       <c r="V46" s="7" t="n"/>
       <c r="Y46" s="7" t="n"/>
       <c r="AB46" s="7" t="n"/>
+      <c r="AC46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="C47" s="7" t="n"/>
@@ -1354,6 +1405,7 @@
       <c r="V47" s="7" t="n"/>
       <c r="Y47" s="7" t="n"/>
       <c r="AB47" s="7" t="n"/>
+      <c r="AC47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="C48" s="7" t="n"/>
@@ -1367,6 +1419,7 @@
       <c r="V48" s="7" t="n"/>
       <c r="Y48" s="7" t="n"/>
       <c r="AB48" s="7" t="n"/>
+      <c r="AC48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="C49" s="7" t="n"/>
@@ -1380,6 +1433,7 @@
       <c r="V49" s="7" t="n"/>
       <c r="Y49" s="7" t="n"/>
       <c r="AB49" s="7" t="n"/>
+      <c r="AC49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="C50" s="7" t="n"/>
@@ -1393,6 +1447,7 @@
       <c r="V50" s="7" t="n"/>
       <c r="Y50" s="7" t="n"/>
       <c r="AB50" s="7" t="n"/>
+      <c r="AC50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="C51" s="7" t="n"/>
@@ -1406,6 +1461,7 @@
       <c r="V51" s="7" t="n"/>
       <c r="Y51" s="7" t="n"/>
       <c r="AB51" s="7" t="n"/>
+      <c r="AC51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="C52" s="7" t="n"/>
@@ -1419,6 +1475,7 @@
       <c r="V52" s="7" t="n"/>
       <c r="Y52" s="7" t="n"/>
       <c r="AB52" s="7" t="n"/>
+      <c r="AC52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="C53" s="7" t="n"/>
@@ -1432,6 +1489,7 @@
       <c r="V53" s="7" t="n"/>
       <c r="Y53" s="7" t="n"/>
       <c r="AB53" s="7" t="n"/>
+      <c r="AC53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="C54" s="7" t="n"/>
@@ -1445,6 +1503,7 @@
       <c r="V54" s="7" t="n"/>
       <c r="Y54" s="7" t="n"/>
       <c r="AB54" s="7" t="n"/>
+      <c r="AC54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="C55" s="7" t="n"/>
@@ -1458,6 +1517,7 @@
       <c r="V55" s="7" t="n"/>
       <c r="Y55" s="7" t="n"/>
       <c r="AB55" s="7" t="n"/>
+      <c r="AC55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="C56" s="7" t="n"/>
@@ -1471,6 +1531,7 @@
       <c r="V56" s="7" t="n"/>
       <c r="Y56" s="7" t="n"/>
       <c r="AB56" s="7" t="n"/>
+      <c r="AC56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="C57" s="7" t="n"/>
@@ -1484,6 +1545,7 @@
       <c r="V57" s="7" t="n"/>
       <c r="Y57" s="7" t="n"/>
       <c r="AB57" s="7" t="n"/>
+      <c r="AC57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="C58" s="7" t="n"/>
@@ -1497,6 +1559,7 @@
       <c r="V58" s="7" t="n"/>
       <c r="Y58" s="7" t="n"/>
       <c r="AB58" s="7" t="n"/>
+      <c r="AC58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="C59" s="7" t="n"/>
@@ -1510,6 +1573,7 @@
       <c r="V59" s="7" t="n"/>
       <c r="Y59" s="7" t="n"/>
       <c r="AB59" s="7" t="n"/>
+      <c r="AC59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="C60" s="7" t="n"/>
@@ -1523,6 +1587,7 @@
       <c r="V60" s="7" t="n"/>
       <c r="Y60" s="7" t="n"/>
       <c r="AB60" s="7" t="n"/>
+      <c r="AC60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="C61" s="7" t="n"/>
@@ -1536,6 +1601,7 @@
       <c r="V61" s="7" t="n"/>
       <c r="Y61" s="7" t="n"/>
       <c r="AB61" s="7" t="n"/>
+      <c r="AC61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="C62" s="7" t="n"/>
@@ -1549,6 +1615,7 @@
       <c r="V62" s="7" t="n"/>
       <c r="Y62" s="7" t="n"/>
       <c r="AB62" s="7" t="n"/>
+      <c r="AC62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="C63" s="7" t="n"/>
@@ -1562,6 +1629,7 @@
       <c r="V63" s="7" t="n"/>
       <c r="Y63" s="7" t="n"/>
       <c r="AB63" s="7" t="n"/>
+      <c r="AC63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="C64" s="7" t="n"/>
@@ -1575,6 +1643,7 @@
       <c r="V64" s="7" t="n"/>
       <c r="Y64" s="7" t="n"/>
       <c r="AB64" s="7" t="n"/>
+      <c r="AC64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="C65" s="7" t="n"/>
@@ -1588,6 +1657,7 @@
       <c r="V65" s="7" t="n"/>
       <c r="Y65" s="7" t="n"/>
       <c r="AB65" s="7" t="n"/>
+      <c r="AC65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="C66" s="7" t="n"/>
@@ -1601,6 +1671,7 @@
       <c r="V66" s="7" t="n"/>
       <c r="Y66" s="7" t="n"/>
       <c r="AB66" s="7" t="n"/>
+      <c r="AC66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="C67" s="7" t="n"/>
@@ -1614,6 +1685,7 @@
       <c r="V67" s="7" t="n"/>
       <c r="Y67" s="7" t="n"/>
       <c r="AB67" s="7" t="n"/>
+      <c r="AC67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="C68" s="7" t="n"/>
@@ -1627,6 +1699,7 @@
       <c r="V68" s="7" t="n"/>
       <c r="Y68" s="7" t="n"/>
       <c r="AB68" s="7" t="n"/>
+      <c r="AC68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="C69" s="7" t="n"/>
@@ -1640,6 +1713,7 @@
       <c r="V69" s="7" t="n"/>
       <c r="Y69" s="7" t="n"/>
       <c r="AB69" s="7" t="n"/>
+      <c r="AC69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="C70" s="7" t="n"/>
@@ -1653,6 +1727,7 @@
       <c r="V70" s="7" t="n"/>
       <c r="Y70" s="7" t="n"/>
       <c r="AB70" s="7" t="n"/>
+      <c r="AC70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="C71" s="7" t="n"/>
@@ -1666,6 +1741,7 @@
       <c r="V71" s="7" t="n"/>
       <c r="Y71" s="7" t="n"/>
       <c r="AB71" s="7" t="n"/>
+      <c r="AC71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="C72" s="7" t="n"/>
@@ -1679,6 +1755,7 @@
       <c r="V72" s="7" t="n"/>
       <c r="Y72" s="7" t="n"/>
       <c r="AB72" s="7" t="n"/>
+      <c r="AC72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="C73" s="7" t="n"/>
@@ -1692,6 +1769,7 @@
       <c r="V73" s="7" t="n"/>
       <c r="Y73" s="7" t="n"/>
       <c r="AB73" s="7" t="n"/>
+      <c r="AC73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="C74" s="7" t="n"/>
@@ -1705,6 +1783,7 @@
       <c r="V74" s="7" t="n"/>
       <c r="Y74" s="7" t="n"/>
       <c r="AB74" s="7" t="n"/>
+      <c r="AC74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="C75" s="7" t="n"/>
@@ -1718,6 +1797,7 @@
       <c r="V75" s="7" t="n"/>
       <c r="Y75" s="7" t="n"/>
       <c r="AB75" s="7" t="n"/>
+      <c r="AC75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="C76" s="7" t="n"/>
@@ -1731,6 +1811,7 @@
       <c r="V76" s="7" t="n"/>
       <c r="Y76" s="7" t="n"/>
       <c r="AB76" s="7" t="n"/>
+      <c r="AC76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="C77" s="7" t="n"/>
@@ -1744,6 +1825,7 @@
       <c r="V77" s="7" t="n"/>
       <c r="Y77" s="7" t="n"/>
       <c r="AB77" s="7" t="n"/>
+      <c r="AC77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="C78" s="7" t="n"/>
@@ -1757,6 +1839,7 @@
       <c r="V78" s="7" t="n"/>
       <c r="Y78" s="7" t="n"/>
       <c r="AB78" s="7" t="n"/>
+      <c r="AC78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="C79" s="7" t="n"/>
@@ -1770,6 +1853,7 @@
       <c r="V79" s="7" t="n"/>
       <c r="Y79" s="7" t="n"/>
       <c r="AB79" s="7" t="n"/>
+      <c r="AC79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="C80" s="7" t="n"/>
@@ -1783,6 +1867,7 @@
       <c r="V80" s="7" t="n"/>
       <c r="Y80" s="7" t="n"/>
       <c r="AB80" s="7" t="n"/>
+      <c r="AC80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="C81" s="7" t="n"/>
@@ -1796,6 +1881,7 @@
       <c r="V81" s="7" t="n"/>
       <c r="Y81" s="7" t="n"/>
       <c r="AB81" s="7" t="n"/>
+      <c r="AC81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="C82" s="7" t="n"/>
@@ -1809,6 +1895,7 @@
       <c r="V82" s="7" t="n"/>
       <c r="Y82" s="7" t="n"/>
       <c r="AB82" s="7" t="n"/>
+      <c r="AC82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="C83" s="7" t="n"/>
@@ -1822,6 +1909,7 @@
       <c r="V83" s="7" t="n"/>
       <c r="Y83" s="7" t="n"/>
       <c r="AB83" s="7" t="n"/>
+      <c r="AC83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="C84" s="7" t="n"/>
@@ -1835,6 +1923,7 @@
       <c r="V84" s="7" t="n"/>
       <c r="Y84" s="7" t="n"/>
       <c r="AB84" s="7" t="n"/>
+      <c r="AC84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="C85" s="7" t="n"/>
@@ -1848,6 +1937,7 @@
       <c r="V85" s="7" t="n"/>
       <c r="Y85" s="7" t="n"/>
       <c r="AB85" s="7" t="n"/>
+      <c r="AC85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="C86" s="7" t="n"/>
@@ -1861,6 +1951,7 @@
       <c r="V86" s="7" t="n"/>
       <c r="Y86" s="7" t="n"/>
       <c r="AB86" s="7" t="n"/>
+      <c r="AC86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="C87" s="7" t="n"/>
@@ -1874,6 +1965,7 @@
       <c r="V87" s="7" t="n"/>
       <c r="Y87" s="7" t="n"/>
       <c r="AB87" s="7" t="n"/>
+      <c r="AC87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="C88" s="7" t="n"/>
@@ -1887,6 +1979,7 @@
       <c r="V88" s="7" t="n"/>
       <c r="Y88" s="7" t="n"/>
       <c r="AB88" s="7" t="n"/>
+      <c r="AC88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="C89" s="7" t="n"/>
@@ -1900,6 +1993,7 @@
       <c r="V89" s="7" t="n"/>
       <c r="Y89" s="7" t="n"/>
       <c r="AB89" s="7" t="n"/>
+      <c r="AC89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="C90" s="7" t="n"/>
@@ -1913,6 +2007,7 @@
       <c r="V90" s="7" t="n"/>
       <c r="Y90" s="7" t="n"/>
       <c r="AB90" s="7" t="n"/>
+      <c r="AC90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="C91" s="7" t="n"/>
@@ -1926,6 +2021,7 @@
       <c r="V91" s="7" t="n"/>
       <c r="Y91" s="7" t="n"/>
       <c r="AB91" s="7" t="n"/>
+      <c r="AC91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="C92" s="7" t="n"/>
@@ -1939,6 +2035,7 @@
       <c r="V92" s="7" t="n"/>
       <c r="Y92" s="7" t="n"/>
       <c r="AB92" s="7" t="n"/>
+      <c r="AC92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="C93" s="7" t="n"/>
@@ -1952,6 +2049,7 @@
       <c r="V93" s="7" t="n"/>
       <c r="Y93" s="7" t="n"/>
       <c r="AB93" s="7" t="n"/>
+      <c r="AC93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="C94" s="7" t="n"/>
@@ -1965,6 +2063,7 @@
       <c r="V94" s="7" t="n"/>
       <c r="Y94" s="7" t="n"/>
       <c r="AB94" s="7" t="n"/>
+      <c r="AC94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="C95" s="7" t="n"/>
@@ -1978,6 +2077,7 @@
       <c r="V95" s="7" t="n"/>
       <c r="Y95" s="7" t="n"/>
       <c r="AB95" s="7" t="n"/>
+      <c r="AC95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="C96" s="7" t="n"/>
@@ -1991,6 +2091,7 @@
       <c r="V96" s="7" t="n"/>
       <c r="Y96" s="7" t="n"/>
       <c r="AB96" s="7" t="n"/>
+      <c r="AC96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="C97" s="7" t="n"/>
@@ -2004,6 +2105,7 @@
       <c r="V97" s="7" t="n"/>
       <c r="Y97" s="7" t="n"/>
       <c r="AB97" s="7" t="n"/>
+      <c r="AC97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="C98" s="7" t="n"/>
@@ -2017,6 +2119,7 @@
       <c r="V98" s="7" t="n"/>
       <c r="Y98" s="7" t="n"/>
       <c r="AB98" s="7" t="n"/>
+      <c r="AC98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="C99" s="7" t="n"/>
@@ -2030,6 +2133,7 @@
       <c r="V99" s="7" t="n"/>
       <c r="Y99" s="7" t="n"/>
       <c r="AB99" s="7" t="n"/>
+      <c r="AC99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="C100" s="7" t="n"/>
@@ -2043,6 +2147,7 @@
       <c r="V100" s="7" t="n"/>
       <c r="Y100" s="7" t="n"/>
       <c r="AB100" s="7" t="n"/>
+      <c r="AC100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="C101" s="7" t="n"/>
@@ -2056,6 +2161,7 @@
       <c r="V101" s="7" t="n"/>
       <c r="Y101" s="7" t="n"/>
       <c r="AB101" s="7" t="n"/>
+      <c r="AC101" s="7" t="n"/>
     </row>
     <row r="102">
       <c r="C102" s="7" t="n"/>
@@ -2069,6 +2175,7 @@
       <c r="V102" s="7" t="n"/>
       <c r="Y102" s="7" t="n"/>
       <c r="AB102" s="7" t="n"/>
+      <c r="AC102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="C103" s="7" t="n"/>
@@ -2082,6 +2189,7 @@
       <c r="V103" s="7" t="n"/>
       <c r="Y103" s="7" t="n"/>
       <c r="AB103" s="7" t="n"/>
+      <c r="AC103" s="7" t="n"/>
     </row>
     <row r="104">
       <c r="C104" s="7" t="n"/>
@@ -2095,6 +2203,7 @@
       <c r="V104" s="7" t="n"/>
       <c r="Y104" s="7" t="n"/>
       <c r="AB104" s="7" t="n"/>
+      <c r="AC104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="C105" s="7" t="n"/>
@@ -2108,6 +2217,7 @@
       <c r="V105" s="7" t="n"/>
       <c r="Y105" s="7" t="n"/>
       <c r="AB105" s="7" t="n"/>
+      <c r="AC105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="C106" s="7" t="n"/>
@@ -2121,6 +2231,7 @@
       <c r="V106" s="7" t="n"/>
       <c r="Y106" s="7" t="n"/>
       <c r="AB106" s="7" t="n"/>
+      <c r="AC106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="C107" s="7" t="n"/>
@@ -2134,6 +2245,7 @@
       <c r="V107" s="7" t="n"/>
       <c r="Y107" s="7" t="n"/>
       <c r="AB107" s="7" t="n"/>
+      <c r="AC107" s="7" t="n"/>
     </row>
     <row r="108">
       <c r="C108" s="7" t="n"/>
@@ -2147,6 +2259,7 @@
       <c r="V108" s="7" t="n"/>
       <c r="Y108" s="7" t="n"/>
       <c r="AB108" s="7" t="n"/>
+      <c r="AC108" s="7" t="n"/>
     </row>
     <row r="109">
       <c r="C109" s="7" t="n"/>
@@ -2160,6 +2273,7 @@
       <c r="V109" s="7" t="n"/>
       <c r="Y109" s="7" t="n"/>
       <c r="AB109" s="7" t="n"/>
+      <c r="AC109" s="7" t="n"/>
     </row>
     <row r="110">
       <c r="C110" s="7" t="n"/>
@@ -2173,6 +2287,7 @@
       <c r="V110" s="7" t="n"/>
       <c r="Y110" s="7" t="n"/>
       <c r="AB110" s="7" t="n"/>
+      <c r="AC110" s="7" t="n"/>
     </row>
     <row r="111">
       <c r="C111" s="7" t="n"/>
@@ -2186,6 +2301,7 @@
       <c r="V111" s="7" t="n"/>
       <c r="Y111" s="7" t="n"/>
       <c r="AB111" s="7" t="n"/>
+      <c r="AC111" s="7" t="n"/>
     </row>
     <row r="112">
       <c r="C112" s="7" t="n"/>
@@ -2199,6 +2315,7 @@
       <c r="V112" s="7" t="n"/>
       <c r="Y112" s="7" t="n"/>
       <c r="AB112" s="7" t="n"/>
+      <c r="AC112" s="7" t="n"/>
     </row>
     <row r="113">
       <c r="C113" s="7" t="n"/>
@@ -2212,6 +2329,7 @@
       <c r="V113" s="7" t="n"/>
       <c r="Y113" s="7" t="n"/>
       <c r="AB113" s="7" t="n"/>
+      <c r="AC113" s="7" t="n"/>
     </row>
     <row r="114">
       <c r="C114" s="7" t="n"/>
@@ -2225,6 +2343,7 @@
       <c r="V114" s="7" t="n"/>
       <c r="Y114" s="7" t="n"/>
       <c r="AB114" s="7" t="n"/>
+      <c r="AC114" s="7" t="n"/>
     </row>
     <row r="115">
       <c r="C115" s="7" t="n"/>
@@ -2238,6 +2357,7 @@
       <c r="V115" s="7" t="n"/>
       <c r="Y115" s="7" t="n"/>
       <c r="AB115" s="7" t="n"/>
+      <c r="AC115" s="7" t="n"/>
     </row>
     <row r="116">
       <c r="C116" s="7" t="n"/>
@@ -2251,6 +2371,7 @@
       <c r="V116" s="7" t="n"/>
       <c r="Y116" s="7" t="n"/>
       <c r="AB116" s="7" t="n"/>
+      <c r="AC116" s="7" t="n"/>
     </row>
     <row r="117">
       <c r="C117" s="7" t="n"/>
@@ -2264,6 +2385,7 @@
       <c r="V117" s="7" t="n"/>
       <c r="Y117" s="7" t="n"/>
       <c r="AB117" s="7" t="n"/>
+      <c r="AC117" s="7" t="n"/>
     </row>
     <row r="118">
       <c r="C118" s="7" t="n"/>
@@ -2277,6 +2399,7 @@
       <c r="V118" s="7" t="n"/>
       <c r="Y118" s="7" t="n"/>
       <c r="AB118" s="7" t="n"/>
+      <c r="AC118" s="7" t="n"/>
     </row>
     <row r="119">
       <c r="C119" s="7" t="n"/>
@@ -2290,6 +2413,7 @@
       <c r="V119" s="7" t="n"/>
       <c r="Y119" s="7" t="n"/>
       <c r="AB119" s="7" t="n"/>
+      <c r="AC119" s="7" t="n"/>
     </row>
     <row r="120">
       <c r="C120" s="7" t="n"/>
@@ -2303,6 +2427,7 @@
       <c r="V120" s="7" t="n"/>
       <c r="Y120" s="7" t="n"/>
       <c r="AB120" s="7" t="n"/>
+      <c r="AC120" s="7" t="n"/>
     </row>
     <row r="121">
       <c r="C121" s="7" t="n"/>
@@ -2316,6 +2441,7 @@
       <c r="V121" s="7" t="n"/>
       <c r="Y121" s="7" t="n"/>
       <c r="AB121" s="7" t="n"/>
+      <c r="AC121" s="7" t="n"/>
     </row>
     <row r="122">
       <c r="C122" s="7" t="n"/>
@@ -2329,6 +2455,7 @@
       <c r="V122" s="7" t="n"/>
       <c r="Y122" s="7" t="n"/>
       <c r="AB122" s="7" t="n"/>
+      <c r="AC122" s="7" t="n"/>
     </row>
     <row r="123">
       <c r="C123" s="7" t="n"/>
@@ -2342,6 +2469,7 @@
       <c r="V123" s="7" t="n"/>
       <c r="Y123" s="7" t="n"/>
       <c r="AB123" s="7" t="n"/>
+      <c r="AC123" s="7" t="n"/>
     </row>
     <row r="124">
       <c r="C124" s="7" t="n"/>
@@ -2355,6 +2483,7 @@
       <c r="V124" s="7" t="n"/>
       <c r="Y124" s="7" t="n"/>
       <c r="AB124" s="7" t="n"/>
+      <c r="AC124" s="7" t="n"/>
     </row>
     <row r="125">
       <c r="C125" s="7" t="n"/>
@@ -2368,6 +2497,7 @@
       <c r="V125" s="7" t="n"/>
       <c r="Y125" s="7" t="n"/>
       <c r="AB125" s="7" t="n"/>
+      <c r="AC125" s="7" t="n"/>
     </row>
     <row r="126">
       <c r="C126" s="7" t="n"/>
@@ -2381,6 +2511,7 @@
       <c r="V126" s="7" t="n"/>
       <c r="Y126" s="7" t="n"/>
       <c r="AB126" s="7" t="n"/>
+      <c r="AC126" s="7" t="n"/>
     </row>
     <row r="127">
       <c r="C127" s="7" t="n"/>
@@ -2394,6 +2525,7 @@
       <c r="V127" s="7" t="n"/>
       <c r="Y127" s="7" t="n"/>
       <c r="AB127" s="7" t="n"/>
+      <c r="AC127" s="7" t="n"/>
     </row>
     <row r="128">
       <c r="C128" s="7" t="n"/>
@@ -2407,6 +2539,7 @@
       <c r="V128" s="7" t="n"/>
       <c r="Y128" s="7" t="n"/>
       <c r="AB128" s="7" t="n"/>
+      <c r="AC128" s="7" t="n"/>
     </row>
     <row r="129">
       <c r="C129" s="7" t="n"/>
@@ -2420,6 +2553,7 @@
       <c r="V129" s="7" t="n"/>
       <c r="Y129" s="7" t="n"/>
       <c r="AB129" s="7" t="n"/>
+      <c r="AC129" s="7" t="n"/>
     </row>
     <row r="130">
       <c r="C130" s="7" t="n"/>
@@ -2433,6 +2567,7 @@
       <c r="V130" s="7" t="n"/>
       <c r="Y130" s="7" t="n"/>
       <c r="AB130" s="7" t="n"/>
+      <c r="AC130" s="7" t="n"/>
     </row>
     <row r="131">
       <c r="C131" s="7" t="n"/>
@@ -2446,6 +2581,7 @@
       <c r="V131" s="7" t="n"/>
       <c r="Y131" s="7" t="n"/>
       <c r="AB131" s="7" t="n"/>
+      <c r="AC131" s="7" t="n"/>
     </row>
     <row r="132">
       <c r="C132" s="7" t="n"/>
@@ -2459,6 +2595,7 @@
       <c r="V132" s="7" t="n"/>
       <c r="Y132" s="7" t="n"/>
       <c r="AB132" s="7" t="n"/>
+      <c r="AC132" s="7" t="n"/>
     </row>
     <row r="133">
       <c r="C133" s="7" t="n"/>
@@ -2472,6 +2609,7 @@
       <c r="V133" s="7" t="n"/>
       <c r="Y133" s="7" t="n"/>
       <c r="AB133" s="7" t="n"/>
+      <c r="AC133" s="7" t="n"/>
     </row>
     <row r="134">
       <c r="C134" s="7" t="n"/>
@@ -2485,6 +2623,7 @@
       <c r="V134" s="7" t="n"/>
       <c r="Y134" s="7" t="n"/>
       <c r="AB134" s="7" t="n"/>
+      <c r="AC134" s="7" t="n"/>
     </row>
     <row r="135">
       <c r="C135" s="7" t="n"/>
@@ -2498,6 +2637,7 @@
       <c r="V135" s="7" t="n"/>
       <c r="Y135" s="7" t="n"/>
       <c r="AB135" s="7" t="n"/>
+      <c r="AC135" s="7" t="n"/>
     </row>
     <row r="136">
       <c r="C136" s="7" t="n"/>
@@ -2511,6 +2651,7 @@
       <c r="V136" s="7" t="n"/>
       <c r="Y136" s="7" t="n"/>
       <c r="AB136" s="7" t="n"/>
+      <c r="AC136" s="7" t="n"/>
     </row>
     <row r="137">
       <c r="C137" s="7" t="n"/>
@@ -2524,6 +2665,7 @@
       <c r="V137" s="7" t="n"/>
       <c r="Y137" s="7" t="n"/>
       <c r="AB137" s="7" t="n"/>
+      <c r="AC137" s="7" t="n"/>
     </row>
     <row r="138">
       <c r="C138" s="7" t="n"/>
@@ -2537,6 +2679,7 @@
       <c r="V138" s="7" t="n"/>
       <c r="Y138" s="7" t="n"/>
       <c r="AB138" s="7" t="n"/>
+      <c r="AC138" s="7" t="n"/>
     </row>
     <row r="139">
       <c r="C139" s="7" t="n"/>
@@ -2550,6 +2693,7 @@
       <c r="V139" s="7" t="n"/>
       <c r="Y139" s="7" t="n"/>
       <c r="AB139" s="7" t="n"/>
+      <c r="AC139" s="7" t="n"/>
     </row>
     <row r="140">
       <c r="C140" s="7" t="n"/>
@@ -2563,6 +2707,7 @@
       <c r="V140" s="7" t="n"/>
       <c r="Y140" s="7" t="n"/>
       <c r="AB140" s="7" t="n"/>
+      <c r="AC140" s="7" t="n"/>
     </row>
     <row r="141">
       <c r="C141" s="7" t="n"/>
@@ -2576,6 +2721,7 @@
       <c r="V141" s="7" t="n"/>
       <c r="Y141" s="7" t="n"/>
       <c r="AB141" s="7" t="n"/>
+      <c r="AC141" s="7" t="n"/>
     </row>
     <row r="142">
       <c r="C142" s="7" t="n"/>
@@ -2589,6 +2735,7 @@
       <c r="V142" s="7" t="n"/>
       <c r="Y142" s="7" t="n"/>
       <c r="AB142" s="7" t="n"/>
+      <c r="AC142" s="7" t="n"/>
     </row>
     <row r="143">
       <c r="C143" s="7" t="n"/>
@@ -2602,6 +2749,7 @@
       <c r="V143" s="7" t="n"/>
       <c r="Y143" s="7" t="n"/>
       <c r="AB143" s="7" t="n"/>
+      <c r="AC143" s="7" t="n"/>
     </row>
     <row r="144">
       <c r="C144" s="7" t="n"/>
@@ -2615,6 +2763,7 @@
       <c r="V144" s="7" t="n"/>
       <c r="Y144" s="7" t="n"/>
       <c r="AB144" s="7" t="n"/>
+      <c r="AC144" s="7" t="n"/>
     </row>
     <row r="145">
       <c r="C145" s="7" t="n"/>
@@ -2628,6 +2777,7 @@
       <c r="V145" s="7" t="n"/>
       <c r="Y145" s="7" t="n"/>
       <c r="AB145" s="7" t="n"/>
+      <c r="AC145" s="7" t="n"/>
     </row>
     <row r="146">
       <c r="C146" s="7" t="n"/>
@@ -2641,6 +2791,7 @@
       <c r="V146" s="7" t="n"/>
       <c r="Y146" s="7" t="n"/>
       <c r="AB146" s="7" t="n"/>
+      <c r="AC146" s="7" t="n"/>
     </row>
     <row r="147">
       <c r="C147" s="7" t="n"/>
@@ -2654,6 +2805,7 @@
       <c r="V147" s="7" t="n"/>
       <c r="Y147" s="7" t="n"/>
       <c r="AB147" s="7" t="n"/>
+      <c r="AC147" s="7" t="n"/>
     </row>
     <row r="148">
       <c r="C148" s="7" t="n"/>
@@ -2667,6 +2819,7 @@
       <c r="V148" s="7" t="n"/>
       <c r="Y148" s="7" t="n"/>
       <c r="AB148" s="7" t="n"/>
+      <c r="AC148" s="7" t="n"/>
     </row>
     <row r="149">
       <c r="C149" s="7" t="n"/>
@@ -2680,6 +2833,7 @@
       <c r="V149" s="7" t="n"/>
       <c r="Y149" s="7" t="n"/>
       <c r="AB149" s="7" t="n"/>
+      <c r="AC149" s="7" t="n"/>
     </row>
     <row r="150">
       <c r="C150" s="7" t="n"/>
@@ -2693,6 +2847,7 @@
       <c r="V150" s="7" t="n"/>
       <c r="Y150" s="7" t="n"/>
       <c r="AB150" s="7" t="n"/>
+      <c r="AC150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="C151" s="7" t="n"/>
@@ -2706,6 +2861,7 @@
       <c r="V151" s="7" t="n"/>
       <c r="Y151" s="7" t="n"/>
       <c r="AB151" s="7" t="n"/>
+      <c r="AC151" s="7" t="n"/>
     </row>
     <row r="152">
       <c r="C152" s="7" t="n"/>
@@ -2719,6 +2875,7 @@
       <c r="V152" s="7" t="n"/>
       <c r="Y152" s="7" t="n"/>
       <c r="AB152" s="7" t="n"/>
+      <c r="AC152" s="7" t="n"/>
     </row>
     <row r="153">
       <c r="C153" s="7" t="n"/>
@@ -2732,6 +2889,7 @@
       <c r="V153" s="7" t="n"/>
       <c r="Y153" s="7" t="n"/>
       <c r="AB153" s="7" t="n"/>
+      <c r="AC153" s="7" t="n"/>
     </row>
     <row r="154">
       <c r="C154" s="7" t="n"/>
@@ -2745,6 +2903,7 @@
       <c r="V154" s="7" t="n"/>
       <c r="Y154" s="7" t="n"/>
       <c r="AB154" s="7" t="n"/>
+      <c r="AC154" s="7" t="n"/>
     </row>
     <row r="155">
       <c r="C155" s="7" t="n"/>
@@ -2758,6 +2917,7 @@
       <c r="V155" s="7" t="n"/>
       <c r="Y155" s="7" t="n"/>
       <c r="AB155" s="7" t="n"/>
+      <c r="AC155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="C156" s="7" t="n"/>
@@ -2771,6 +2931,7 @@
       <c r="V156" s="7" t="n"/>
       <c r="Y156" s="7" t="n"/>
       <c r="AB156" s="7" t="n"/>
+      <c r="AC156" s="7" t="n"/>
     </row>
     <row r="157">
       <c r="C157" s="7" t="n"/>
@@ -2784,6 +2945,7 @@
       <c r="V157" s="7" t="n"/>
       <c r="Y157" s="7" t="n"/>
       <c r="AB157" s="7" t="n"/>
+      <c r="AC157" s="7" t="n"/>
     </row>
     <row r="158">
       <c r="C158" s="7" t="n"/>
@@ -2797,6 +2959,7 @@
       <c r="V158" s="7" t="n"/>
       <c r="Y158" s="7" t="n"/>
       <c r="AB158" s="7" t="n"/>
+      <c r="AC158" s="7" t="n"/>
     </row>
     <row r="159">
       <c r="C159" s="7" t="n"/>
@@ -2810,6 +2973,7 @@
       <c r="V159" s="7" t="n"/>
       <c r="Y159" s="7" t="n"/>
       <c r="AB159" s="7" t="n"/>
+      <c r="AC159" s="7" t="n"/>
     </row>
     <row r="160">
       <c r="C160" s="7" t="n"/>
@@ -2823,6 +2987,7 @@
       <c r="V160" s="7" t="n"/>
       <c r="Y160" s="7" t="n"/>
       <c r="AB160" s="7" t="n"/>
+      <c r="AC160" s="7" t="n"/>
     </row>
     <row r="161">
       <c r="C161" s="7" t="n"/>
@@ -2836,6 +3001,7 @@
       <c r="V161" s="7" t="n"/>
       <c r="Y161" s="7" t="n"/>
       <c r="AB161" s="7" t="n"/>
+      <c r="AC161" s="7" t="n"/>
     </row>
     <row r="162">
       <c r="C162" s="7" t="n"/>
@@ -2849,6 +3015,7 @@
       <c r="V162" s="7" t="n"/>
       <c r="Y162" s="7" t="n"/>
       <c r="AB162" s="7" t="n"/>
+      <c r="AC162" s="7" t="n"/>
     </row>
     <row r="163">
       <c r="C163" s="7" t="n"/>
@@ -2862,6 +3029,7 @@
       <c r="V163" s="7" t="n"/>
       <c r="Y163" s="7" t="n"/>
       <c r="AB163" s="7" t="n"/>
+      <c r="AC163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="C164" s="7" t="n"/>
@@ -2875,6 +3043,7 @@
       <c r="V164" s="7" t="n"/>
       <c r="Y164" s="7" t="n"/>
       <c r="AB164" s="7" t="n"/>
+      <c r="AC164" s="7" t="n"/>
     </row>
     <row r="165">
       <c r="C165" s="7" t="n"/>
@@ -2888,6 +3057,7 @@
       <c r="V165" s="7" t="n"/>
       <c r="Y165" s="7" t="n"/>
       <c r="AB165" s="7" t="n"/>
+      <c r="AC165" s="7" t="n"/>
     </row>
     <row r="166">
       <c r="C166" s="7" t="n"/>
@@ -2901,6 +3071,7 @@
       <c r="V166" s="7" t="n"/>
       <c r="Y166" s="7" t="n"/>
       <c r="AB166" s="7" t="n"/>
+      <c r="AC166" s="7" t="n"/>
     </row>
     <row r="167">
       <c r="C167" s="7" t="n"/>
@@ -2914,6 +3085,7 @@
       <c r="V167" s="7" t="n"/>
       <c r="Y167" s="7" t="n"/>
       <c r="AB167" s="7" t="n"/>
+      <c r="AC167" s="7" t="n"/>
     </row>
     <row r="168">
       <c r="C168" s="7" t="n"/>
@@ -2927,6 +3099,7 @@
       <c r="V168" s="7" t="n"/>
       <c r="Y168" s="7" t="n"/>
       <c r="AB168" s="7" t="n"/>
+      <c r="AC168" s="7" t="n"/>
     </row>
     <row r="169">
       <c r="C169" s="7" t="n"/>
@@ -2940,6 +3113,7 @@
       <c r="V169" s="7" t="n"/>
       <c r="Y169" s="7" t="n"/>
       <c r="AB169" s="7" t="n"/>
+      <c r="AC169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="C170" s="7" t="n"/>
@@ -2953,6 +3127,7 @@
       <c r="V170" s="7" t="n"/>
       <c r="Y170" s="7" t="n"/>
       <c r="AB170" s="7" t="n"/>
+      <c r="AC170" s="7" t="n"/>
     </row>
     <row r="171">
       <c r="C171" s="7" t="n"/>
@@ -2966,6 +3141,7 @@
       <c r="V171" s="7" t="n"/>
       <c r="Y171" s="7" t="n"/>
       <c r="AB171" s="7" t="n"/>
+      <c r="AC171" s="7" t="n"/>
     </row>
     <row r="172">
       <c r="C172" s="7" t="n"/>
@@ -2979,6 +3155,7 @@
       <c r="V172" s="7" t="n"/>
       <c r="Y172" s="7" t="n"/>
       <c r="AB172" s="7" t="n"/>
+      <c r="AC172" s="7" t="n"/>
     </row>
     <row r="173">
       <c r="C173" s="7" t="n"/>
@@ -2992,6 +3169,7 @@
       <c r="V173" s="7" t="n"/>
       <c r="Y173" s="7" t="n"/>
       <c r="AB173" s="7" t="n"/>
+      <c r="AC173" s="7" t="n"/>
     </row>
     <row r="174">
       <c r="C174" s="7" t="n"/>
@@ -3005,6 +3183,7 @@
       <c r="V174" s="7" t="n"/>
       <c r="Y174" s="7" t="n"/>
       <c r="AB174" s="7" t="n"/>
+      <c r="AC174" s="7" t="n"/>
     </row>
     <row r="175">
       <c r="C175" s="7" t="n"/>
@@ -3018,6 +3197,7 @@
       <c r="V175" s="7" t="n"/>
       <c r="Y175" s="7" t="n"/>
       <c r="AB175" s="7" t="n"/>
+      <c r="AC175" s="7" t="n"/>
     </row>
     <row r="176">
       <c r="C176" s="7" t="n"/>
@@ -3031,6 +3211,7 @@
       <c r="V176" s="7" t="n"/>
       <c r="Y176" s="7" t="n"/>
       <c r="AB176" s="7" t="n"/>
+      <c r="AC176" s="7" t="n"/>
     </row>
     <row r="177">
       <c r="C177" s="7" t="n"/>
@@ -3044,6 +3225,7 @@
       <c r="V177" s="7" t="n"/>
       <c r="Y177" s="7" t="n"/>
       <c r="AB177" s="7" t="n"/>
+      <c r="AC177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="C178" s="7" t="n"/>
@@ -3057,6 +3239,7 @@
       <c r="V178" s="7" t="n"/>
       <c r="Y178" s="7" t="n"/>
       <c r="AB178" s="7" t="n"/>
+      <c r="AC178" s="7" t="n"/>
     </row>
     <row r="179">
       <c r="C179" s="7" t="n"/>
@@ -3070,6 +3253,7 @@
       <c r="V179" s="7" t="n"/>
       <c r="Y179" s="7" t="n"/>
       <c r="AB179" s="7" t="n"/>
+      <c r="AC179" s="7" t="n"/>
     </row>
     <row r="180">
       <c r="C180" s="7" t="n"/>
@@ -3083,6 +3267,7 @@
       <c r="V180" s="7" t="n"/>
       <c r="Y180" s="7" t="n"/>
       <c r="AB180" s="7" t="n"/>
+      <c r="AC180" s="7" t="n"/>
     </row>
     <row r="181">
       <c r="C181" s="7" t="n"/>
@@ -3096,6 +3281,7 @@
       <c r="V181" s="7" t="n"/>
       <c r="Y181" s="7" t="n"/>
       <c r="AB181" s="7" t="n"/>
+      <c r="AC181" s="7" t="n"/>
     </row>
     <row r="182">
       <c r="C182" s="7" t="n"/>
@@ -3109,6 +3295,7 @@
       <c r="V182" s="7" t="n"/>
       <c r="Y182" s="7" t="n"/>
       <c r="AB182" s="7" t="n"/>
+      <c r="AC182" s="7" t="n"/>
     </row>
     <row r="183">
       <c r="C183" s="7" t="n"/>
@@ -3122,6 +3309,7 @@
       <c r="V183" s="7" t="n"/>
       <c r="Y183" s="7" t="n"/>
       <c r="AB183" s="7" t="n"/>
+      <c r="AC183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="C184" s="7" t="n"/>
@@ -3135,6 +3323,7 @@
       <c r="V184" s="7" t="n"/>
       <c r="Y184" s="7" t="n"/>
       <c r="AB184" s="7" t="n"/>
+      <c r="AC184" s="7" t="n"/>
     </row>
     <row r="185">
       <c r="C185" s="7" t="n"/>
@@ -3148,6 +3337,7 @@
       <c r="V185" s="7" t="n"/>
       <c r="Y185" s="7" t="n"/>
       <c r="AB185" s="7" t="n"/>
+      <c r="AC185" s="7" t="n"/>
     </row>
     <row r="186">
       <c r="C186" s="7" t="n"/>
@@ -3161,6 +3351,7 @@
       <c r="V186" s="7" t="n"/>
       <c r="Y186" s="7" t="n"/>
       <c r="AB186" s="7" t="n"/>
+      <c r="AC186" s="7" t="n"/>
     </row>
     <row r="187">
       <c r="C187" s="7" t="n"/>
@@ -3174,6 +3365,7 @@
       <c r="V187" s="7" t="n"/>
       <c r="Y187" s="7" t="n"/>
       <c r="AB187" s="7" t="n"/>
+      <c r="AC187" s="7" t="n"/>
     </row>
     <row r="188">
       <c r="C188" s="7" t="n"/>
@@ -3187,6 +3379,7 @@
       <c r="V188" s="7" t="n"/>
       <c r="Y188" s="7" t="n"/>
       <c r="AB188" s="7" t="n"/>
+      <c r="AC188" s="7" t="n"/>
     </row>
     <row r="189">
       <c r="C189" s="7" t="n"/>
@@ -3200,6 +3393,7 @@
       <c r="V189" s="7" t="n"/>
       <c r="Y189" s="7" t="n"/>
       <c r="AB189" s="7" t="n"/>
+      <c r="AC189" s="7" t="n"/>
     </row>
     <row r="190">
       <c r="C190" s="7" t="n"/>
@@ -3213,6 +3407,7 @@
       <c r="V190" s="7" t="n"/>
       <c r="Y190" s="7" t="n"/>
       <c r="AB190" s="7" t="n"/>
+      <c r="AC190" s="7" t="n"/>
     </row>
     <row r="191">
       <c r="C191" s="7" t="n"/>
@@ -3226,6 +3421,7 @@
       <c r="V191" s="7" t="n"/>
       <c r="Y191" s="7" t="n"/>
       <c r="AB191" s="7" t="n"/>
+      <c r="AC191" s="7" t="n"/>
     </row>
     <row r="192">
       <c r="C192" s="7" t="n"/>
@@ -3239,6 +3435,7 @@
       <c r="V192" s="7" t="n"/>
       <c r="Y192" s="7" t="n"/>
       <c r="AB192" s="7" t="n"/>
+      <c r="AC192" s="7" t="n"/>
     </row>
     <row r="193">
       <c r="C193" s="7" t="n"/>
@@ -3252,6 +3449,7 @@
       <c r="V193" s="7" t="n"/>
       <c r="Y193" s="7" t="n"/>
       <c r="AB193" s="7" t="n"/>
+      <c r="AC193" s="7" t="n"/>
     </row>
     <row r="194">
       <c r="C194" s="7" t="n"/>
@@ -3265,6 +3463,7 @@
       <c r="V194" s="7" t="n"/>
       <c r="Y194" s="7" t="n"/>
       <c r="AB194" s="7" t="n"/>
+      <c r="AC194" s="7" t="n"/>
     </row>
     <row r="195">
       <c r="C195" s="7" t="n"/>
@@ -3278,6 +3477,7 @@
       <c r="V195" s="7" t="n"/>
       <c r="Y195" s="7" t="n"/>
       <c r="AB195" s="7" t="n"/>
+      <c r="AC195" s="7" t="n"/>
     </row>
     <row r="196">
       <c r="C196" s="7" t="n"/>
@@ -3291,6 +3491,7 @@
       <c r="V196" s="7" t="n"/>
       <c r="Y196" s="7" t="n"/>
       <c r="AB196" s="7" t="n"/>
+      <c r="AC196" s="7" t="n"/>
     </row>
     <row r="197">
       <c r="C197" s="7" t="n"/>
@@ -3304,6 +3505,7 @@
       <c r="V197" s="7" t="n"/>
       <c r="Y197" s="7" t="n"/>
       <c r="AB197" s="7" t="n"/>
+      <c r="AC197" s="7" t="n"/>
     </row>
     <row r="198">
       <c r="C198" s="7" t="n"/>
@@ -3317,6 +3519,7 @@
       <c r="V198" s="7" t="n"/>
       <c r="Y198" s="7" t="n"/>
       <c r="AB198" s="7" t="n"/>
+      <c r="AC198" s="7" t="n"/>
     </row>
     <row r="199">
       <c r="C199" s="7" t="n"/>
@@ -3330,6 +3533,7 @@
       <c r="V199" s="7" t="n"/>
       <c r="Y199" s="7" t="n"/>
       <c r="AB199" s="7" t="n"/>
+      <c r="AC199" s="7" t="n"/>
     </row>
     <row r="200">
       <c r="C200" s="7" t="n"/>
@@ -3343,6 +3547,7 @@
       <c r="V200" s="7" t="n"/>
       <c r="Y200" s="7" t="n"/>
       <c r="AB200" s="7" t="n"/>
+      <c r="AC200" s="7" t="n"/>
     </row>
     <row r="201">
       <c r="C201" s="7" t="n"/>
@@ -3356,6 +3561,7 @@
       <c r="V201" s="7" t="n"/>
       <c r="Y201" s="7" t="n"/>
       <c r="AB201" s="7" t="n"/>
+      <c r="AC201" s="7" t="n"/>
     </row>
     <row r="202">
       <c r="C202" s="7" t="n"/>
@@ -3369,6 +3575,7 @@
       <c r="V202" s="7" t="n"/>
       <c r="Y202" s="7" t="n"/>
       <c r="AB202" s="7" t="n"/>
+      <c r="AC202" s="7" t="n"/>
     </row>
     <row r="203">
       <c r="C203" s="7" t="n"/>
@@ -3382,6 +3589,7 @@
       <c r="V203" s="7" t="n"/>
       <c r="Y203" s="7" t="n"/>
       <c r="AB203" s="7" t="n"/>
+      <c r="AC203" s="7" t="n"/>
     </row>
     <row r="204">
       <c r="C204" s="7" t="n"/>
@@ -3395,6 +3603,7 @@
       <c r="V204" s="7" t="n"/>
       <c r="Y204" s="7" t="n"/>
       <c r="AB204" s="7" t="n"/>
+      <c r="AC204" s="7" t="n"/>
     </row>
     <row r="205">
       <c r="C205" s="7" t="n"/>
@@ -3408,6 +3617,7 @@
       <c r="V205" s="7" t="n"/>
       <c r="Y205" s="7" t="n"/>
       <c r="AB205" s="7" t="n"/>
+      <c r="AC205" s="7" t="n"/>
     </row>
     <row r="206">
       <c r="C206" s="7" t="n"/>
@@ -3421,6 +3631,7 @@
       <c r="V206" s="7" t="n"/>
       <c r="Y206" s="7" t="n"/>
       <c r="AB206" s="7" t="n"/>
+      <c r="AC206" s="7" t="n"/>
     </row>
     <row r="207">
       <c r="C207" s="7" t="n"/>
@@ -3434,6 +3645,7 @@
       <c r="V207" s="7" t="n"/>
       <c r="Y207" s="7" t="n"/>
       <c r="AB207" s="7" t="n"/>
+      <c r="AC207" s="7" t="n"/>
     </row>
     <row r="208">
       <c r="C208" s="7" t="n"/>
@@ -3447,6 +3659,7 @@
       <c r="V208" s="7" t="n"/>
       <c r="Y208" s="7" t="n"/>
       <c r="AB208" s="7" t="n"/>
+      <c r="AC208" s="7" t="n"/>
     </row>
     <row r="209">
       <c r="C209" s="7" t="n"/>
@@ -3460,6 +3673,7 @@
       <c r="V209" s="7" t="n"/>
       <c r="Y209" s="7" t="n"/>
       <c r="AB209" s="7" t="n"/>
+      <c r="AC209" s="7" t="n"/>
     </row>
     <row r="210">
       <c r="C210" s="7" t="n"/>
@@ -3473,6 +3687,7 @@
       <c r="V210" s="7" t="n"/>
       <c r="Y210" s="7" t="n"/>
       <c r="AB210" s="7" t="n"/>
+      <c r="AC210" s="7" t="n"/>
     </row>
     <row r="211">
       <c r="C211" s="7" t="n"/>
@@ -3486,6 +3701,7 @@
       <c r="V211" s="7" t="n"/>
       <c r="Y211" s="7" t="n"/>
       <c r="AB211" s="7" t="n"/>
+      <c r="AC211" s="7" t="n"/>
     </row>
     <row r="212">
       <c r="C212" s="7" t="n"/>
@@ -3499,6 +3715,7 @@
       <c r="V212" s="7" t="n"/>
       <c r="Y212" s="7" t="n"/>
       <c r="AB212" s="7" t="n"/>
+      <c r="AC212" s="7" t="n"/>
     </row>
     <row r="213">
       <c r="C213" s="7" t="n"/>
@@ -3512,6 +3729,7 @@
       <c r="V213" s="7" t="n"/>
       <c r="Y213" s="7" t="n"/>
       <c r="AB213" s="7" t="n"/>
+      <c r="AC213" s="7" t="n"/>
     </row>
     <row r="214">
       <c r="C214" s="7" t="n"/>
@@ -3525,6 +3743,7 @@
       <c r="V214" s="7" t="n"/>
       <c r="Y214" s="7" t="n"/>
       <c r="AB214" s="7" t="n"/>
+      <c r="AC214" s="7" t="n"/>
     </row>
     <row r="215">
       <c r="C215" s="7" t="n"/>
@@ -3538,6 +3757,7 @@
       <c r="V215" s="7" t="n"/>
       <c r="Y215" s="7" t="n"/>
       <c r="AB215" s="7" t="n"/>
+      <c r="AC215" s="7" t="n"/>
     </row>
     <row r="216">
       <c r="C216" s="7" t="n"/>
@@ -3551,6 +3771,7 @@
       <c r="V216" s="7" t="n"/>
       <c r="Y216" s="7" t="n"/>
       <c r="AB216" s="7" t="n"/>
+      <c r="AC216" s="7" t="n"/>
     </row>
     <row r="217">
       <c r="C217" s="7" t="n"/>
@@ -3564,6 +3785,7 @@
       <c r="V217" s="7" t="n"/>
       <c r="Y217" s="7" t="n"/>
       <c r="AB217" s="7" t="n"/>
+      <c r="AC217" s="7" t="n"/>
     </row>
     <row r="218">
       <c r="C218" s="7" t="n"/>
@@ -3577,6 +3799,7 @@
       <c r="V218" s="7" t="n"/>
       <c r="Y218" s="7" t="n"/>
       <c r="AB218" s="7" t="n"/>
+      <c r="AC218" s="7" t="n"/>
     </row>
     <row r="219">
       <c r="C219" s="7" t="n"/>
@@ -3590,6 +3813,7 @@
       <c r="V219" s="7" t="n"/>
       <c r="Y219" s="7" t="n"/>
       <c r="AB219" s="7" t="n"/>
+      <c r="AC219" s="7" t="n"/>
     </row>
     <row r="220">
       <c r="C220" s="7" t="n"/>
@@ -3603,6 +3827,7 @@
       <c r="V220" s="7" t="n"/>
       <c r="Y220" s="7" t="n"/>
       <c r="AB220" s="7" t="n"/>
+      <c r="AC220" s="7" t="n"/>
     </row>
     <row r="221">
       <c r="C221" s="7" t="n"/>
@@ -3616,6 +3841,7 @@
       <c r="V221" s="7" t="n"/>
       <c r="Y221" s="7" t="n"/>
       <c r="AB221" s="7" t="n"/>
+      <c r="AC221" s="7" t="n"/>
     </row>
     <row r="222">
       <c r="C222" s="7" t="n"/>
@@ -3629,6 +3855,7 @@
       <c r="V222" s="7" t="n"/>
       <c r="Y222" s="7" t="n"/>
       <c r="AB222" s="7" t="n"/>
+      <c r="AC222" s="7" t="n"/>
     </row>
     <row r="223">
       <c r="C223" s="7" t="n"/>
@@ -3642,6 +3869,7 @@
       <c r="V223" s="7" t="n"/>
       <c r="Y223" s="7" t="n"/>
       <c r="AB223" s="7" t="n"/>
+      <c r="AC223" s="7" t="n"/>
     </row>
     <row r="224">
       <c r="C224" s="7" t="n"/>
@@ -3655,6 +3883,7 @@
       <c r="V224" s="7" t="n"/>
       <c r="Y224" s="7" t="n"/>
       <c r="AB224" s="7" t="n"/>
+      <c r="AC224" s="7" t="n"/>
     </row>
     <row r="225">
       <c r="C225" s="7" t="n"/>
@@ -3668,6 +3897,7 @@
       <c r="V225" s="7" t="n"/>
       <c r="Y225" s="7" t="n"/>
       <c r="AB225" s="7" t="n"/>
+      <c r="AC225" s="7" t="n"/>
     </row>
     <row r="226">
       <c r="C226" s="7" t="n"/>
@@ -3681,6 +3911,7 @@
       <c r="V226" s="7" t="n"/>
       <c r="Y226" s="7" t="n"/>
       <c r="AB226" s="7" t="n"/>
+      <c r="AC226" s="7" t="n"/>
     </row>
     <row r="227">
       <c r="C227" s="7" t="n"/>
@@ -3694,6 +3925,7 @@
       <c r="V227" s="7" t="n"/>
       <c r="Y227" s="7" t="n"/>
       <c r="AB227" s="7" t="n"/>
+      <c r="AC227" s="7" t="n"/>
     </row>
     <row r="228">
       <c r="C228" s="7" t="n"/>
@@ -3707,6 +3939,7 @@
       <c r="V228" s="7" t="n"/>
       <c r="Y228" s="7" t="n"/>
       <c r="AB228" s="7" t="n"/>
+      <c r="AC228" s="7" t="n"/>
     </row>
     <row r="229">
       <c r="C229" s="7" t="n"/>
@@ -3720,6 +3953,7 @@
       <c r="V229" s="7" t="n"/>
       <c r="Y229" s="7" t="n"/>
       <c r="AB229" s="7" t="n"/>
+      <c r="AC229" s="7" t="n"/>
     </row>
     <row r="230">
       <c r="C230" s="7" t="n"/>
@@ -3733,6 +3967,7 @@
       <c r="V230" s="7" t="n"/>
       <c r="Y230" s="7" t="n"/>
       <c r="AB230" s="7" t="n"/>
+      <c r="AC230" s="7" t="n"/>
     </row>
     <row r="231">
       <c r="C231" s="7" t="n"/>
@@ -3746,6 +3981,7 @@
       <c r="V231" s="7" t="n"/>
       <c r="Y231" s="7" t="n"/>
       <c r="AB231" s="7" t="n"/>
+      <c r="AC231" s="7" t="n"/>
     </row>
     <row r="232">
       <c r="C232" s="7" t="n"/>
@@ -3759,6 +3995,7 @@
       <c r="V232" s="7" t="n"/>
       <c r="Y232" s="7" t="n"/>
       <c r="AB232" s="7" t="n"/>
+      <c r="AC232" s="7" t="n"/>
     </row>
     <row r="233">
       <c r="C233" s="7" t="n"/>
@@ -3772,6 +4009,7 @@
       <c r="V233" s="7" t="n"/>
       <c r="Y233" s="7" t="n"/>
       <c r="AB233" s="7" t="n"/>
+      <c r="AC233" s="7" t="n"/>
     </row>
     <row r="234">
       <c r="C234" s="7" t="n"/>
@@ -3785,6 +4023,7 @@
       <c r="V234" s="7" t="n"/>
       <c r="Y234" s="7" t="n"/>
       <c r="AB234" s="7" t="n"/>
+      <c r="AC234" s="7" t="n"/>
     </row>
     <row r="235">
       <c r="C235" s="7" t="n"/>
@@ -3798,6 +4037,7 @@
       <c r="V235" s="7" t="n"/>
       <c r="Y235" s="7" t="n"/>
       <c r="AB235" s="7" t="n"/>
+      <c r="AC235" s="7" t="n"/>
     </row>
     <row r="236">
       <c r="C236" s="7" t="n"/>
@@ -3811,6 +4051,7 @@
       <c r="V236" s="7" t="n"/>
       <c r="Y236" s="7" t="n"/>
       <c r="AB236" s="7" t="n"/>
+      <c r="AC236" s="7" t="n"/>
     </row>
     <row r="237">
       <c r="C237" s="7" t="n"/>
@@ -3824,6 +4065,7 @@
       <c r="V237" s="7" t="n"/>
       <c r="Y237" s="7" t="n"/>
       <c r="AB237" s="7" t="n"/>
+      <c r="AC237" s="7" t="n"/>
     </row>
     <row r="238">
       <c r="C238" s="7" t="n"/>
@@ -3837,6 +4079,7 @@
       <c r="V238" s="7" t="n"/>
       <c r="Y238" s="7" t="n"/>
       <c r="AB238" s="7" t="n"/>
+      <c r="AC238" s="7" t="n"/>
     </row>
     <row r="239">
       <c r="C239" s="7" t="n"/>
@@ -3850,6 +4093,7 @@
       <c r="V239" s="7" t="n"/>
       <c r="Y239" s="7" t="n"/>
       <c r="AB239" s="7" t="n"/>
+      <c r="AC239" s="7" t="n"/>
     </row>
     <row r="240">
       <c r="C240" s="7" t="n"/>
@@ -3863,6 +4107,7 @@
       <c r="V240" s="7" t="n"/>
       <c r="Y240" s="7" t="n"/>
       <c r="AB240" s="7" t="n"/>
+      <c r="AC240" s="7" t="n"/>
     </row>
     <row r="241">
       <c r="C241" s="7" t="n"/>
@@ -3876,6 +4121,7 @@
       <c r="V241" s="7" t="n"/>
       <c r="Y241" s="7" t="n"/>
       <c r="AB241" s="7" t="n"/>
+      <c r="AC241" s="7" t="n"/>
     </row>
     <row r="242">
       <c r="C242" s="7" t="n"/>
@@ -3889,6 +4135,7 @@
       <c r="V242" s="7" t="n"/>
       <c r="Y242" s="7" t="n"/>
       <c r="AB242" s="7" t="n"/>
+      <c r="AC242" s="7" t="n"/>
     </row>
     <row r="243">
       <c r="C243" s="7" t="n"/>
@@ -3902,6 +4149,7 @@
       <c r="V243" s="7" t="n"/>
       <c r="Y243" s="7" t="n"/>
       <c r="AB243" s="7" t="n"/>
+      <c r="AC243" s="7" t="n"/>
     </row>
     <row r="244">
       <c r="C244" s="7" t="n"/>
@@ -3915,6 +4163,7 @@
       <c r="V244" s="7" t="n"/>
       <c r="Y244" s="7" t="n"/>
       <c r="AB244" s="7" t="n"/>
+      <c r="AC244" s="7" t="n"/>
     </row>
     <row r="245">
       <c r="C245" s="7" t="n"/>
@@ -3928,6 +4177,7 @@
       <c r="V245" s="7" t="n"/>
       <c r="Y245" s="7" t="n"/>
       <c r="AB245" s="7" t="n"/>
+      <c r="AC245" s="7" t="n"/>
     </row>
     <row r="246">
       <c r="C246" s="7" t="n"/>
@@ -3941,6 +4191,7 @@
       <c r="V246" s="7" t="n"/>
       <c r="Y246" s="7" t="n"/>
       <c r="AB246" s="7" t="n"/>
+      <c r="AC246" s="7" t="n"/>
     </row>
     <row r="247">
       <c r="C247" s="7" t="n"/>
@@ -3954,6 +4205,7 @@
       <c r="V247" s="7" t="n"/>
       <c r="Y247" s="7" t="n"/>
       <c r="AB247" s="7" t="n"/>
+      <c r="AC247" s="7" t="n"/>
     </row>
     <row r="248">
       <c r="C248" s="7" t="n"/>
@@ -3967,6 +4219,7 @@
       <c r="V248" s="7" t="n"/>
       <c r="Y248" s="7" t="n"/>
       <c r="AB248" s="7" t="n"/>
+      <c r="AC248" s="7" t="n"/>
     </row>
     <row r="249">
       <c r="C249" s="7" t="n"/>
@@ -3980,6 +4233,7 @@
       <c r="V249" s="7" t="n"/>
       <c r="Y249" s="7" t="n"/>
       <c r="AB249" s="7" t="n"/>
+      <c r="AC249" s="7" t="n"/>
     </row>
     <row r="250">
       <c r="C250" s="7" t="n"/>
@@ -3993,6 +4247,7 @@
       <c r="V250" s="7" t="n"/>
       <c r="Y250" s="7" t="n"/>
       <c r="AB250" s="7" t="n"/>
+      <c r="AC250" s="7" t="n"/>
     </row>
     <row r="251">
       <c r="C251" s="7" t="n"/>
@@ -4006,6 +4261,7 @@
       <c r="V251" s="7" t="n"/>
       <c r="Y251" s="7" t="n"/>
       <c r="AB251" s="7" t="n"/>
+      <c r="AC251" s="7" t="n"/>
     </row>
     <row r="252">
       <c r="C252" s="7" t="n"/>
@@ -4019,6 +4275,7 @@
       <c r="V252" s="7" t="n"/>
       <c r="Y252" s="7" t="n"/>
       <c r="AB252" s="7" t="n"/>
+      <c r="AC252" s="7" t="n"/>
     </row>
     <row r="253">
       <c r="C253" s="7" t="n"/>
@@ -4032,6 +4289,7 @@
       <c r="V253" s="7" t="n"/>
       <c r="Y253" s="7" t="n"/>
       <c r="AB253" s="7" t="n"/>
+      <c r="AC253" s="7" t="n"/>
     </row>
     <row r="254">
       <c r="C254" s="7" t="n"/>
@@ -4045,6 +4303,7 @@
       <c r="V254" s="7" t="n"/>
       <c r="Y254" s="7" t="n"/>
       <c r="AB254" s="7" t="n"/>
+      <c r="AC254" s="7" t="n"/>
     </row>
     <row r="255">
       <c r="C255" s="7" t="n"/>
@@ -4058,6 +4317,7 @@
       <c r="V255" s="7" t="n"/>
       <c r="Y255" s="7" t="n"/>
       <c r="AB255" s="7" t="n"/>
+      <c r="AC255" s="7" t="n"/>
     </row>
     <row r="256">
       <c r="C256" s="7" t="n"/>
@@ -4071,6 +4331,7 @@
       <c r="V256" s="7" t="n"/>
       <c r="Y256" s="7" t="n"/>
       <c r="AB256" s="7" t="n"/>
+      <c r="AC256" s="7" t="n"/>
     </row>
     <row r="257">
       <c r="C257" s="7" t="n"/>
@@ -4084,6 +4345,7 @@
       <c r="V257" s="7" t="n"/>
       <c r="Y257" s="7" t="n"/>
       <c r="AB257" s="7" t="n"/>
+      <c r="AC257" s="7" t="n"/>
     </row>
     <row r="258">
       <c r="C258" s="7" t="n"/>
@@ -4097,6 +4359,7 @@
       <c r="V258" s="7" t="n"/>
       <c r="Y258" s="7" t="n"/>
       <c r="AB258" s="7" t="n"/>
+      <c r="AC258" s="7" t="n"/>
     </row>
     <row r="259">
       <c r="C259" s="7" t="n"/>
@@ -4110,6 +4373,7 @@
       <c r="V259" s="7" t="n"/>
       <c r="Y259" s="7" t="n"/>
       <c r="AB259" s="7" t="n"/>
+      <c r="AC259" s="7" t="n"/>
     </row>
     <row r="260">
       <c r="C260" s="7" t="n"/>
@@ -4123,6 +4387,7 @@
       <c r="V260" s="7" t="n"/>
       <c r="Y260" s="7" t="n"/>
       <c r="AB260" s="7" t="n"/>
+      <c r="AC260" s="7" t="n"/>
     </row>
     <row r="261">
       <c r="C261" s="7" t="n"/>
@@ -4136,6 +4401,7 @@
       <c r="V261" s="7" t="n"/>
       <c r="Y261" s="7" t="n"/>
       <c r="AB261" s="7" t="n"/>
+      <c r="AC261" s="7" t="n"/>
     </row>
     <row r="262">
       <c r="C262" s="7" t="n"/>
@@ -4149,6 +4415,7 @@
       <c r="V262" s="7" t="n"/>
       <c r="Y262" s="7" t="n"/>
       <c r="AB262" s="7" t="n"/>
+      <c r="AC262" s="7" t="n"/>
     </row>
     <row r="263">
       <c r="C263" s="7" t="n"/>
@@ -4162,6 +4429,7 @@
       <c r="V263" s="7" t="n"/>
       <c r="Y263" s="7" t="n"/>
       <c r="AB263" s="7" t="n"/>
+      <c r="AC263" s="7" t="n"/>
     </row>
     <row r="264">
       <c r="C264" s="7" t="n"/>
@@ -4175,6 +4443,7 @@
       <c r="V264" s="7" t="n"/>
       <c r="Y264" s="7" t="n"/>
       <c r="AB264" s="7" t="n"/>
+      <c r="AC264" s="7" t="n"/>
     </row>
     <row r="265">
       <c r="C265" s="7" t="n"/>
@@ -4188,6 +4457,7 @@
       <c r="V265" s="7" t="n"/>
       <c r="Y265" s="7" t="n"/>
       <c r="AB265" s="7" t="n"/>
+      <c r="AC265" s="7" t="n"/>
     </row>
     <row r="266">
       <c r="C266" s="7" t="n"/>
@@ -4201,6 +4471,7 @@
       <c r="V266" s="7" t="n"/>
       <c r="Y266" s="7" t="n"/>
       <c r="AB266" s="7" t="n"/>
+      <c r="AC266" s="7" t="n"/>
     </row>
     <row r="267">
       <c r="C267" s="7" t="n"/>
@@ -4214,6 +4485,7 @@
       <c r="V267" s="7" t="n"/>
       <c r="Y267" s="7" t="n"/>
       <c r="AB267" s="7" t="n"/>
+      <c r="AC267" s="7" t="n"/>
     </row>
     <row r="268">
       <c r="C268" s="7" t="n"/>
@@ -4227,6 +4499,7 @@
       <c r="V268" s="7" t="n"/>
       <c r="Y268" s="7" t="n"/>
       <c r="AB268" s="7" t="n"/>
+      <c r="AC268" s="7" t="n"/>
     </row>
     <row r="269">
       <c r="C269" s="7" t="n"/>
@@ -4240,6 +4513,7 @@
       <c r="V269" s="7" t="n"/>
       <c r="Y269" s="7" t="n"/>
       <c r="AB269" s="7" t="n"/>
+      <c r="AC269" s="7" t="n"/>
     </row>
     <row r="270">
       <c r="C270" s="7" t="n"/>
@@ -4253,6 +4527,7 @@
       <c r="V270" s="7" t="n"/>
       <c r="Y270" s="7" t="n"/>
       <c r="AB270" s="7" t="n"/>
+      <c r="AC270" s="7" t="n"/>
     </row>
     <row r="271">
       <c r="C271" s="7" t="n"/>
@@ -4266,6 +4541,7 @@
       <c r="V271" s="7" t="n"/>
       <c r="Y271" s="7" t="n"/>
       <c r="AB271" s="7" t="n"/>
+      <c r="AC271" s="7" t="n"/>
     </row>
     <row r="272">
       <c r="C272" s="7" t="n"/>
@@ -4279,6 +4555,7 @@
       <c r="V272" s="7" t="n"/>
       <c r="Y272" s="7" t="n"/>
       <c r="AB272" s="7" t="n"/>
+      <c r="AC272" s="7" t="n"/>
     </row>
     <row r="273">
       <c r="C273" s="7" t="n"/>
@@ -4292,6 +4569,7 @@
       <c r="V273" s="7" t="n"/>
       <c r="Y273" s="7" t="n"/>
       <c r="AB273" s="7" t="n"/>
+      <c r="AC273" s="7" t="n"/>
     </row>
     <row r="274">
       <c r="C274" s="7" t="n"/>
@@ -4305,6 +4583,7 @@
       <c r="V274" s="7" t="n"/>
       <c r="Y274" s="7" t="n"/>
       <c r="AB274" s="7" t="n"/>
+      <c r="AC274" s="7" t="n"/>
     </row>
     <row r="275">
       <c r="C275" s="7" t="n"/>
@@ -4318,6 +4597,7 @@
       <c r="V275" s="7" t="n"/>
       <c r="Y275" s="7" t="n"/>
       <c r="AB275" s="7" t="n"/>
+      <c r="AC275" s="7" t="n"/>
     </row>
     <row r="276">
       <c r="C276" s="7" t="n"/>
@@ -4331,6 +4611,7 @@
       <c r="V276" s="7" t="n"/>
       <c r="Y276" s="7" t="n"/>
       <c r="AB276" s="7" t="n"/>
+      <c r="AC276" s="7" t="n"/>
     </row>
     <row r="277">
       <c r="C277" s="7" t="n"/>
@@ -4344,6 +4625,7 @@
       <c r="V277" s="7" t="n"/>
       <c r="Y277" s="7" t="n"/>
       <c r="AB277" s="7" t="n"/>
+      <c r="AC277" s="7" t="n"/>
     </row>
     <row r="278">
       <c r="C278" s="7" t="n"/>
@@ -4357,6 +4639,7 @@
       <c r="V278" s="7" t="n"/>
       <c r="Y278" s="7" t="n"/>
       <c r="AB278" s="7" t="n"/>
+      <c r="AC278" s="7" t="n"/>
     </row>
     <row r="279">
       <c r="C279" s="7" t="n"/>
@@ -4370,6 +4653,7 @@
       <c r="V279" s="7" t="n"/>
       <c r="Y279" s="7" t="n"/>
       <c r="AB279" s="7" t="n"/>
+      <c r="AC279" s="7" t="n"/>
     </row>
     <row r="280">
       <c r="C280" s="7" t="n"/>
@@ -4383,6 +4667,7 @@
       <c r="V280" s="7" t="n"/>
       <c r="Y280" s="7" t="n"/>
       <c r="AB280" s="7" t="n"/>
+      <c r="AC280" s="7" t="n"/>
     </row>
     <row r="281">
       <c r="C281" s="7" t="n"/>
@@ -4396,6 +4681,7 @@
       <c r="V281" s="7" t="n"/>
       <c r="Y281" s="7" t="n"/>
       <c r="AB281" s="7" t="n"/>
+      <c r="AC281" s="7" t="n"/>
     </row>
     <row r="282">
       <c r="C282" s="7" t="n"/>
@@ -4409,6 +4695,7 @@
       <c r="V282" s="7" t="n"/>
       <c r="Y282" s="7" t="n"/>
       <c r="AB282" s="7" t="n"/>
+      <c r="AC282" s="7" t="n"/>
     </row>
     <row r="283">
       <c r="C283" s="7" t="n"/>
@@ -4422,6 +4709,7 @@
       <c r="V283" s="7" t="n"/>
       <c r="Y283" s="7" t="n"/>
       <c r="AB283" s="7" t="n"/>
+      <c r="AC283" s="7" t="n"/>
     </row>
     <row r="284">
       <c r="C284" s="7" t="n"/>
@@ -4435,6 +4723,7 @@
       <c r="V284" s="7" t="n"/>
       <c r="Y284" s="7" t="n"/>
       <c r="AB284" s="7" t="n"/>
+      <c r="AC284" s="7" t="n"/>
     </row>
     <row r="285">
       <c r="C285" s="7" t="n"/>
@@ -4448,6 +4737,7 @@
       <c r="V285" s="7" t="n"/>
       <c r="Y285" s="7" t="n"/>
       <c r="AB285" s="7" t="n"/>
+      <c r="AC285" s="7" t="n"/>
     </row>
     <row r="286">
       <c r="C286" s="7" t="n"/>
@@ -4461,6 +4751,7 @@
       <c r="V286" s="7" t="n"/>
       <c r="Y286" s="7" t="n"/>
       <c r="AB286" s="7" t="n"/>
+      <c r="AC286" s="7" t="n"/>
     </row>
     <row r="287">
       <c r="C287" s="7" t="n"/>
@@ -4474,6 +4765,7 @@
       <c r="V287" s="7" t="n"/>
       <c r="Y287" s="7" t="n"/>
       <c r="AB287" s="7" t="n"/>
+      <c r="AC287" s="7" t="n"/>
     </row>
     <row r="288">
       <c r="C288" s="7" t="n"/>
@@ -4487,6 +4779,7 @@
       <c r="V288" s="7" t="n"/>
       <c r="Y288" s="7" t="n"/>
       <c r="AB288" s="7" t="n"/>
+      <c r="AC288" s="7" t="n"/>
     </row>
     <row r="289">
       <c r="C289" s="7" t="n"/>
@@ -4500,6 +4793,7 @@
       <c r="V289" s="7" t="n"/>
       <c r="Y289" s="7" t="n"/>
       <c r="AB289" s="7" t="n"/>
+      <c r="AC289" s="7" t="n"/>
     </row>
     <row r="290">
       <c r="C290" s="7" t="n"/>
@@ -4513,6 +4807,7 @@
       <c r="V290" s="7" t="n"/>
       <c r="Y290" s="7" t="n"/>
       <c r="AB290" s="7" t="n"/>
+      <c r="AC290" s="7" t="n"/>
     </row>
     <row r="291">
       <c r="C291" s="7" t="n"/>
@@ -4526,6 +4821,7 @@
       <c r="V291" s="7" t="n"/>
       <c r="Y291" s="7" t="n"/>
       <c r="AB291" s="7" t="n"/>
+      <c r="AC291" s="7" t="n"/>
     </row>
     <row r="292">
       <c r="C292" s="7" t="n"/>
@@ -4539,6 +4835,7 @@
       <c r="V292" s="7" t="n"/>
       <c r="Y292" s="7" t="n"/>
       <c r="AB292" s="7" t="n"/>
+      <c r="AC292" s="7" t="n"/>
     </row>
     <row r="293">
       <c r="C293" s="7" t="n"/>
@@ -4552,6 +4849,7 @@
       <c r="V293" s="7" t="n"/>
       <c r="Y293" s="7" t="n"/>
       <c r="AB293" s="7" t="n"/>
+      <c r="AC293" s="7" t="n"/>
     </row>
     <row r="294">
       <c r="C294" s="7" t="n"/>
@@ -4565,6 +4863,7 @@
       <c r="V294" s="7" t="n"/>
       <c r="Y294" s="7" t="n"/>
       <c r="AB294" s="7" t="n"/>
+      <c r="AC294" s="7" t="n"/>
     </row>
     <row r="295">
       <c r="C295" s="7" t="n"/>
@@ -4578,6 +4877,7 @@
       <c r="V295" s="7" t="n"/>
       <c r="Y295" s="7" t="n"/>
       <c r="AB295" s="7" t="n"/>
+      <c r="AC295" s="7" t="n"/>
     </row>
     <row r="296">
       <c r="C296" s="7" t="n"/>
@@ -4591,6 +4891,7 @@
       <c r="V296" s="7" t="n"/>
       <c r="Y296" s="7" t="n"/>
       <c r="AB296" s="7" t="n"/>
+      <c r="AC296" s="7" t="n"/>
     </row>
     <row r="297">
       <c r="C297" s="7" t="n"/>
@@ -4604,6 +4905,7 @@
       <c r="V297" s="7" t="n"/>
       <c r="Y297" s="7" t="n"/>
       <c r="AB297" s="7" t="n"/>
+      <c r="AC297" s="7" t="n"/>
     </row>
     <row r="298">
       <c r="C298" s="7" t="n"/>
@@ -4617,6 +4919,7 @@
       <c r="V298" s="7" t="n"/>
       <c r="Y298" s="7" t="n"/>
       <c r="AB298" s="7" t="n"/>
+      <c r="AC298" s="7" t="n"/>
     </row>
     <row r="299">
       <c r="C299" s="7" t="n"/>
@@ -4630,6 +4933,7 @@
       <c r="V299" s="7" t="n"/>
       <c r="Y299" s="7" t="n"/>
       <c r="AB299" s="7" t="n"/>
+      <c r="AC299" s="7" t="n"/>
     </row>
     <row r="300">
       <c r="C300" s="7" t="n"/>
@@ -4643,6 +4947,7 @@
       <c r="V300" s="7" t="n"/>
       <c r="Y300" s="7" t="n"/>
       <c r="AB300" s="7" t="n"/>
+      <c r="AC300" s="7" t="n"/>
     </row>
     <row r="301">
       <c r="C301" s="7" t="n"/>
@@ -4656,6 +4961,7 @@
       <c r="V301" s="7" t="n"/>
       <c r="Y301" s="7" t="n"/>
       <c r="AB301" s="7" t="n"/>
+      <c r="AC301" s="7" t="n"/>
     </row>
     <row r="302">
       <c r="C302" s="7" t="n"/>
@@ -4669,6 +4975,7 @@
       <c r="V302" s="7" t="n"/>
       <c r="Y302" s="7" t="n"/>
       <c r="AB302" s="7" t="n"/>
+      <c r="AC302" s="7" t="n"/>
     </row>
     <row r="303">
       <c r="C303" s="7" t="n"/>
@@ -4682,6 +4989,7 @@
       <c r="V303" s="7" t="n"/>
       <c r="Y303" s="7" t="n"/>
       <c r="AB303" s="7" t="n"/>
+      <c r="AC303" s="7" t="n"/>
     </row>
     <row r="304">
       <c r="C304" s="7" t="n"/>
@@ -4695,6 +5003,7 @@
       <c r="V304" s="7" t="n"/>
       <c r="Y304" s="7" t="n"/>
       <c r="AB304" s="7" t="n"/>
+      <c r="AC304" s="7" t="n"/>
     </row>
     <row r="305">
       <c r="C305" s="7" t="n"/>
@@ -4708,6 +5017,7 @@
       <c r="V305" s="7" t="n"/>
       <c r="Y305" s="7" t="n"/>
       <c r="AB305" s="7" t="n"/>
+      <c r="AC305" s="7" t="n"/>
     </row>
     <row r="306">
       <c r="C306" s="7" t="n"/>
@@ -4721,6 +5031,7 @@
       <c r="V306" s="7" t="n"/>
       <c r="Y306" s="7" t="n"/>
       <c r="AB306" s="7" t="n"/>
+      <c r="AC306" s="7" t="n"/>
     </row>
     <row r="307">
       <c r="C307" s="7" t="n"/>
@@ -4734,6 +5045,7 @@
       <c r="V307" s="7" t="n"/>
       <c r="Y307" s="7" t="n"/>
       <c r="AB307" s="7" t="n"/>
+      <c r="AC307" s="7" t="n"/>
     </row>
     <row r="308">
       <c r="C308" s="7" t="n"/>
@@ -4747,6 +5059,7 @@
       <c r="V308" s="7" t="n"/>
       <c r="Y308" s="7" t="n"/>
       <c r="AB308" s="7" t="n"/>
+      <c r="AC308" s="7" t="n"/>
     </row>
     <row r="309">
       <c r="C309" s="7" t="n"/>
@@ -4760,6 +5073,7 @@
       <c r="V309" s="7" t="n"/>
       <c r="Y309" s="7" t="n"/>
       <c r="AB309" s="7" t="n"/>
+      <c r="AC309" s="7" t="n"/>
     </row>
     <row r="310">
       <c r="C310" s="7" t="n"/>
@@ -4773,6 +5087,7 @@
       <c r="V310" s="7" t="n"/>
       <c r="Y310" s="7" t="n"/>
       <c r="AB310" s="7" t="n"/>
+      <c r="AC310" s="7" t="n"/>
     </row>
     <row r="311">
       <c r="C311" s="7" t="n"/>
@@ -4786,6 +5101,7 @@
       <c r="V311" s="7" t="n"/>
       <c r="Y311" s="7" t="n"/>
       <c r="AB311" s="7" t="n"/>
+      <c r="AC311" s="7" t="n"/>
     </row>
     <row r="312">
       <c r="C312" s="7" t="n"/>
@@ -4799,6 +5115,7 @@
       <c r="V312" s="7" t="n"/>
       <c r="Y312" s="7" t="n"/>
       <c r="AB312" s="7" t="n"/>
+      <c r="AC312" s="7" t="n"/>
     </row>
     <row r="313">
       <c r="C313" s="7" t="n"/>
@@ -4812,6 +5129,7 @@
       <c r="V313" s="7" t="n"/>
       <c r="Y313" s="7" t="n"/>
       <c r="AB313" s="7" t="n"/>
+      <c r="AC313" s="7" t="n"/>
     </row>
     <row r="314">
       <c r="C314" s="7" t="n"/>
@@ -4825,6 +5143,7 @@
       <c r="V314" s="7" t="n"/>
       <c r="Y314" s="7" t="n"/>
       <c r="AB314" s="7" t="n"/>
+      <c r="AC314" s="7" t="n"/>
     </row>
     <row r="315">
       <c r="C315" s="7" t="n"/>
@@ -4838,6 +5157,7 @@
       <c r="V315" s="7" t="n"/>
       <c r="Y315" s="7" t="n"/>
       <c r="AB315" s="7" t="n"/>
+      <c r="AC315" s="7" t="n"/>
     </row>
     <row r="316">
       <c r="C316" s="7" t="n"/>
@@ -4851,6 +5171,7 @@
       <c r="V316" s="7" t="n"/>
       <c r="Y316" s="7" t="n"/>
       <c r="AB316" s="7" t="n"/>
+      <c r="AC316" s="7" t="n"/>
     </row>
     <row r="317">
       <c r="C317" s="7" t="n"/>
@@ -4864,6 +5185,7 @@
       <c r="V317" s="7" t="n"/>
       <c r="Y317" s="7" t="n"/>
       <c r="AB317" s="7" t="n"/>
+      <c r="AC317" s="7" t="n"/>
     </row>
     <row r="318">
       <c r="C318" s="7" t="n"/>
@@ -4877,6 +5199,7 @@
       <c r="V318" s="7" t="n"/>
       <c r="Y318" s="7" t="n"/>
       <c r="AB318" s="7" t="n"/>
+      <c r="AC318" s="7" t="n"/>
     </row>
     <row r="319">
       <c r="C319" s="7" t="n"/>
@@ -4890,6 +5213,7 @@
       <c r="V319" s="7" t="n"/>
       <c r="Y319" s="7" t="n"/>
       <c r="AB319" s="7" t="n"/>
+      <c r="AC319" s="7" t="n"/>
     </row>
     <row r="320">
       <c r="C320" s="7" t="n"/>
@@ -4903,6 +5227,7 @@
       <c r="V320" s="7" t="n"/>
       <c r="Y320" s="7" t="n"/>
       <c r="AB320" s="7" t="n"/>
+      <c r="AC320" s="7" t="n"/>
     </row>
     <row r="321">
       <c r="C321" s="7" t="n"/>
@@ -4916,6 +5241,7 @@
       <c r="V321" s="7" t="n"/>
       <c r="Y321" s="7" t="n"/>
       <c r="AB321" s="7" t="n"/>
+      <c r="AC321" s="7" t="n"/>
     </row>
     <row r="322">
       <c r="C322" s="7" t="n"/>
@@ -4929,6 +5255,7 @@
       <c r="V322" s="7" t="n"/>
       <c r="Y322" s="7" t="n"/>
       <c r="AB322" s="7" t="n"/>
+      <c r="AC322" s="7" t="n"/>
     </row>
     <row r="323">
       <c r="C323" s="7" t="n"/>
@@ -4942,6 +5269,7 @@
       <c r="V323" s="7" t="n"/>
       <c r="Y323" s="7" t="n"/>
       <c r="AB323" s="7" t="n"/>
+      <c r="AC323" s="7" t="n"/>
     </row>
     <row r="324">
       <c r="C324" s="7" t="n"/>
@@ -4955,6 +5283,7 @@
       <c r="V324" s="7" t="n"/>
       <c r="Y324" s="7" t="n"/>
       <c r="AB324" s="7" t="n"/>
+      <c r="AC324" s="7" t="n"/>
     </row>
     <row r="325">
       <c r="C325" s="7" t="n"/>
@@ -4968,6 +5297,7 @@
       <c r="V325" s="7" t="n"/>
       <c r="Y325" s="7" t="n"/>
       <c r="AB325" s="7" t="n"/>
+      <c r="AC325" s="7" t="n"/>
     </row>
     <row r="326">
       <c r="C326" s="7" t="n"/>
@@ -4981,6 +5311,7 @@
       <c r="V326" s="7" t="n"/>
       <c r="Y326" s="7" t="n"/>
       <c r="AB326" s="7" t="n"/>
+      <c r="AC326" s="7" t="n"/>
     </row>
     <row r="327">
       <c r="C327" s="7" t="n"/>
@@ -4994,6 +5325,7 @@
       <c r="V327" s="7" t="n"/>
       <c r="Y327" s="7" t="n"/>
       <c r="AB327" s="7" t="n"/>
+      <c r="AC327" s="7" t="n"/>
     </row>
     <row r="328">
       <c r="C328" s="7" t="n"/>
@@ -5007,6 +5339,7 @@
       <c r="V328" s="7" t="n"/>
       <c r="Y328" s="7" t="n"/>
       <c r="AB328" s="7" t="n"/>
+      <c r="AC328" s="7" t="n"/>
     </row>
     <row r="329">
       <c r="C329" s="7" t="n"/>
@@ -5020,6 +5353,7 @@
       <c r="V329" s="7" t="n"/>
       <c r="Y329" s="7" t="n"/>
       <c r="AB329" s="7" t="n"/>
+      <c r="AC329" s="7" t="n"/>
     </row>
     <row r="330">
       <c r="C330" s="7" t="n"/>
@@ -5033,6 +5367,7 @@
       <c r="V330" s="7" t="n"/>
       <c r="Y330" s="7" t="n"/>
       <c r="AB330" s="7" t="n"/>
+      <c r="AC330" s="7" t="n"/>
     </row>
     <row r="331">
       <c r="C331" s="7" t="n"/>
@@ -5046,6 +5381,7 @@
       <c r="V331" s="7" t="n"/>
       <c r="Y331" s="7" t="n"/>
       <c r="AB331" s="7" t="n"/>
+      <c r="AC331" s="7" t="n"/>
     </row>
     <row r="332">
       <c r="C332" s="7" t="n"/>
@@ -5059,6 +5395,7 @@
       <c r="V332" s="7" t="n"/>
       <c r="Y332" s="7" t="n"/>
       <c r="AB332" s="7" t="n"/>
+      <c r="AC332" s="7" t="n"/>
     </row>
     <row r="333">
       <c r="C333" s="7" t="n"/>
@@ -5072,6 +5409,7 @@
       <c r="V333" s="7" t="n"/>
       <c r="Y333" s="7" t="n"/>
       <c r="AB333" s="7" t="n"/>
+      <c r="AC333" s="7" t="n"/>
     </row>
     <row r="334">
       <c r="C334" s="7" t="n"/>
@@ -5085,6 +5423,7 @@
       <c r="V334" s="7" t="n"/>
       <c r="Y334" s="7" t="n"/>
       <c r="AB334" s="7" t="n"/>
+      <c r="AC334" s="7" t="n"/>
     </row>
     <row r="335">
       <c r="C335" s="7" t="n"/>
@@ -5098,6 +5437,7 @@
       <c r="V335" s="7" t="n"/>
       <c r="Y335" s="7" t="n"/>
       <c r="AB335" s="7" t="n"/>
+      <c r="AC335" s="7" t="n"/>
     </row>
     <row r="336">
       <c r="C336" s="7" t="n"/>
@@ -5111,6 +5451,7 @@
       <c r="V336" s="7" t="n"/>
       <c r="Y336" s="7" t="n"/>
       <c r="AB336" s="7" t="n"/>
+      <c r="AC336" s="7" t="n"/>
     </row>
     <row r="337">
       <c r="C337" s="7" t="n"/>
@@ -5124,6 +5465,7 @@
       <c r="V337" s="7" t="n"/>
       <c r="Y337" s="7" t="n"/>
       <c r="AB337" s="7" t="n"/>
+      <c r="AC337" s="7" t="n"/>
     </row>
     <row r="338">
       <c r="C338" s="7" t="n"/>
@@ -5137,6 +5479,7 @@
       <c r="V338" s="7" t="n"/>
       <c r="Y338" s="7" t="n"/>
       <c r="AB338" s="7" t="n"/>
+      <c r="AC338" s="7" t="n"/>
     </row>
     <row r="339">
       <c r="C339" s="7" t="n"/>
@@ -5150,6 +5493,7 @@
       <c r="V339" s="7" t="n"/>
       <c r="Y339" s="7" t="n"/>
       <c r="AB339" s="7" t="n"/>
+      <c r="AC339" s="7" t="n"/>
     </row>
     <row r="340">
       <c r="C340" s="7" t="n"/>
@@ -5163,6 +5507,7 @@
       <c r="V340" s="7" t="n"/>
       <c r="Y340" s="7" t="n"/>
       <c r="AB340" s="7" t="n"/>
+      <c r="AC340" s="7" t="n"/>
     </row>
     <row r="341">
       <c r="C341" s="7" t="n"/>
@@ -5176,6 +5521,7 @@
       <c r="V341" s="7" t="n"/>
       <c r="Y341" s="7" t="n"/>
       <c r="AB341" s="7" t="n"/>
+      <c r="AC341" s="7" t="n"/>
     </row>
     <row r="342">
       <c r="C342" s="7" t="n"/>
@@ -5189,6 +5535,7 @@
       <c r="V342" s="7" t="n"/>
       <c r="Y342" s="7" t="n"/>
       <c r="AB342" s="7" t="n"/>
+      <c r="AC342" s="7" t="n"/>
     </row>
     <row r="343">
       <c r="C343" s="7" t="n"/>
@@ -5202,6 +5549,7 @@
       <c r="V343" s="7" t="n"/>
       <c r="Y343" s="7" t="n"/>
       <c r="AB343" s="7" t="n"/>
+      <c r="AC343" s="7" t="n"/>
     </row>
     <row r="344">
       <c r="C344" s="7" t="n"/>
@@ -5215,6 +5563,7 @@
       <c r="V344" s="7" t="n"/>
       <c r="Y344" s="7" t="n"/>
       <c r="AB344" s="7" t="n"/>
+      <c r="AC344" s="7" t="n"/>
     </row>
     <row r="345">
       <c r="C345" s="7" t="n"/>
@@ -5228,6 +5577,7 @@
       <c r="V345" s="7" t="n"/>
       <c r="Y345" s="7" t="n"/>
       <c r="AB345" s="7" t="n"/>
+      <c r="AC345" s="7" t="n"/>
     </row>
     <row r="346">
       <c r="C346" s="7" t="n"/>
@@ -5241,6 +5591,7 @@
       <c r="V346" s="7" t="n"/>
       <c r="Y346" s="7" t="n"/>
       <c r="AB346" s="7" t="n"/>
+      <c r="AC346" s="7" t="n"/>
     </row>
     <row r="347">
       <c r="C347" s="7" t="n"/>
@@ -5254,6 +5605,7 @@
       <c r="V347" s="7" t="n"/>
       <c r="Y347" s="7" t="n"/>
       <c r="AB347" s="7" t="n"/>
+      <c r="AC347" s="7" t="n"/>
     </row>
     <row r="348">
       <c r="C348" s="7" t="n"/>
@@ -5267,6 +5619,7 @@
       <c r="V348" s="7" t="n"/>
       <c r="Y348" s="7" t="n"/>
       <c r="AB348" s="7" t="n"/>
+      <c r="AC348" s="7" t="n"/>
     </row>
     <row r="349">
       <c r="C349" s="7" t="n"/>
@@ -5280,6 +5633,7 @@
       <c r="V349" s="7" t="n"/>
       <c r="Y349" s="7" t="n"/>
       <c r="AB349" s="7" t="n"/>
+      <c r="AC349" s="7" t="n"/>
     </row>
     <row r="350">
       <c r="C350" s="7" t="n"/>
@@ -5293,6 +5647,7 @@
       <c r="V350" s="7" t="n"/>
       <c r="Y350" s="7" t="n"/>
       <c r="AB350" s="7" t="n"/>
+      <c r="AC350" s="7" t="n"/>
     </row>
     <row r="351">
       <c r="C351" s="7" t="n"/>
@@ -5306,6 +5661,7 @@
       <c r="V351" s="7" t="n"/>
       <c r="Y351" s="7" t="n"/>
       <c r="AB351" s="7" t="n"/>
+      <c r="AC351" s="7" t="n"/>
     </row>
     <row r="352">
       <c r="C352" s="7" t="n"/>
@@ -5319,6 +5675,7 @@
       <c r="V352" s="7" t="n"/>
       <c r="Y352" s="7" t="n"/>
       <c r="AB352" s="7" t="n"/>
+      <c r="AC352" s="7" t="n"/>
     </row>
     <row r="353">
       <c r="C353" s="7" t="n"/>
@@ -5332,6 +5689,7 @@
       <c r="V353" s="7" t="n"/>
       <c r="Y353" s="7" t="n"/>
       <c r="AB353" s="7" t="n"/>
+      <c r="AC353" s="7" t="n"/>
     </row>
     <row r="354">
       <c r="C354" s="7" t="n"/>
@@ -5345,6 +5703,7 @@
       <c r="V354" s="7" t="n"/>
       <c r="Y354" s="7" t="n"/>
       <c r="AB354" s="7" t="n"/>
+      <c r="AC354" s="7" t="n"/>
     </row>
     <row r="355">
       <c r="C355" s="7" t="n"/>
@@ -5358,6 +5717,7 @@
       <c r="V355" s="7" t="n"/>
       <c r="Y355" s="7" t="n"/>
       <c r="AB355" s="7" t="n"/>
+      <c r="AC355" s="7" t="n"/>
     </row>
     <row r="356">
       <c r="C356" s="7" t="n"/>
@@ -5371,6 +5731,7 @@
       <c r="V356" s="7" t="n"/>
       <c r="Y356" s="7" t="n"/>
       <c r="AB356" s="7" t="n"/>
+      <c r="AC356" s="7" t="n"/>
     </row>
     <row r="357">
       <c r="C357" s="7" t="n"/>
@@ -5384,6 +5745,7 @@
       <c r="V357" s="7" t="n"/>
       <c r="Y357" s="7" t="n"/>
       <c r="AB357" s="7" t="n"/>
+      <c r="AC357" s="7" t="n"/>
     </row>
     <row r="358">
       <c r="C358" s="7" t="n"/>
@@ -5397,6 +5759,7 @@
       <c r="V358" s="7" t="n"/>
       <c r="Y358" s="7" t="n"/>
       <c r="AB358" s="7" t="n"/>
+      <c r="AC358" s="7" t="n"/>
     </row>
     <row r="359">
       <c r="C359" s="7" t="n"/>
@@ -5410,6 +5773,7 @@
       <c r="V359" s="7" t="n"/>
       <c r="Y359" s="7" t="n"/>
       <c r="AB359" s="7" t="n"/>
+      <c r="AC359" s="7" t="n"/>
     </row>
     <row r="360">
       <c r="C360" s="7" t="n"/>
@@ -5423,6 +5787,7 @@
       <c r="V360" s="7" t="n"/>
       <c r="Y360" s="7" t="n"/>
       <c r="AB360" s="7" t="n"/>
+      <c r="AC360" s="7" t="n"/>
     </row>
     <row r="361">
       <c r="C361" s="7" t="n"/>
@@ -5436,6 +5801,7 @@
       <c r="V361" s="7" t="n"/>
       <c r="Y361" s="7" t="n"/>
       <c r="AB361" s="7" t="n"/>
+      <c r="AC361" s="7" t="n"/>
     </row>
     <row r="362">
       <c r="C362" s="7" t="n"/>
@@ -5449,6 +5815,7 @@
       <c r="V362" s="7" t="n"/>
       <c r="Y362" s="7" t="n"/>
       <c r="AB362" s="7" t="n"/>
+      <c r="AC362" s="7" t="n"/>
     </row>
     <row r="363">
       <c r="C363" s="7" t="n"/>
@@ -5462,6 +5829,7 @@
       <c r="V363" s="7" t="n"/>
       <c r="Y363" s="7" t="n"/>
       <c r="AB363" s="7" t="n"/>
+      <c r="AC363" s="7" t="n"/>
     </row>
     <row r="364">
       <c r="C364" s="7" t="n"/>
@@ -5475,6 +5843,7 @@
       <c r="V364" s="7" t="n"/>
       <c r="Y364" s="7" t="n"/>
       <c r="AB364" s="7" t="n"/>
+      <c r="AC364" s="7" t="n"/>
     </row>
     <row r="365">
       <c r="C365" s="7" t="n"/>
@@ -5488,6 +5857,7 @@
       <c r="V365" s="7" t="n"/>
       <c r="Y365" s="7" t="n"/>
       <c r="AB365" s="7" t="n"/>
+      <c r="AC365" s="7" t="n"/>
     </row>
     <row r="366">
       <c r="C366" s="7" t="n"/>
@@ -5501,6 +5871,7 @@
       <c r="V366" s="7" t="n"/>
       <c r="Y366" s="7" t="n"/>
       <c r="AB366" s="7" t="n"/>
+      <c r="AC366" s="7" t="n"/>
     </row>
     <row r="367">
       <c r="C367" s="7" t="n"/>
@@ -5514,6 +5885,7 @@
       <c r="V367" s="7" t="n"/>
       <c r="Y367" s="7" t="n"/>
       <c r="AB367" s="7" t="n"/>
+      <c r="AC367" s="7" t="n"/>
     </row>
     <row r="368">
       <c r="C368" s="7" t="n"/>
@@ -5527,6 +5899,7 @@
       <c r="V368" s="7" t="n"/>
       <c r="Y368" s="7" t="n"/>
       <c r="AB368" s="7" t="n"/>
+      <c r="AC368" s="7" t="n"/>
     </row>
     <row r="369">
       <c r="C369" s="7" t="n"/>
@@ -5540,6 +5913,7 @@
       <c r="V369" s="7" t="n"/>
       <c r="Y369" s="7" t="n"/>
       <c r="AB369" s="7" t="n"/>
+      <c r="AC369" s="7" t="n"/>
     </row>
     <row r="370">
       <c r="C370" s="7" t="n"/>
@@ -5553,6 +5927,7 @@
       <c r="V370" s="7" t="n"/>
       <c r="Y370" s="7" t="n"/>
       <c r="AB370" s="7" t="n"/>
+      <c r="AC370" s="7" t="n"/>
     </row>
     <row r="371">
       <c r="C371" s="7" t="n"/>
@@ -5566,6 +5941,7 @@
       <c r="V371" s="7" t="n"/>
       <c r="Y371" s="7" t="n"/>
       <c r="AB371" s="7" t="n"/>
+      <c r="AC371" s="7" t="n"/>
     </row>
     <row r="372">
       <c r="C372" s="7" t="n"/>
@@ -5579,6 +5955,7 @@
       <c r="V372" s="7" t="n"/>
       <c r="Y372" s="7" t="n"/>
       <c r="AB372" s="7" t="n"/>
+      <c r="AC372" s="7" t="n"/>
     </row>
     <row r="373">
       <c r="C373" s="7" t="n"/>
@@ -5592,6 +5969,7 @@
       <c r="V373" s="7" t="n"/>
       <c r="Y373" s="7" t="n"/>
       <c r="AB373" s="7" t="n"/>
+      <c r="AC373" s="7" t="n"/>
     </row>
     <row r="374">
       <c r="C374" s="7" t="n"/>
@@ -5605,6 +5983,7 @@
       <c r="V374" s="7" t="n"/>
       <c r="Y374" s="7" t="n"/>
       <c r="AB374" s="7" t="n"/>
+      <c r="AC374" s="7" t="n"/>
     </row>
     <row r="375">
       <c r="C375" s="7" t="n"/>
@@ -5618,6 +5997,7 @@
       <c r="V375" s="7" t="n"/>
       <c r="Y375" s="7" t="n"/>
       <c r="AB375" s="7" t="n"/>
+      <c r="AC375" s="7" t="n"/>
     </row>
     <row r="376">
       <c r="C376" s="7" t="n"/>
@@ -5631,6 +6011,7 @@
       <c r="V376" s="7" t="n"/>
       <c r="Y376" s="7" t="n"/>
       <c r="AB376" s="7" t="n"/>
+      <c r="AC376" s="7" t="n"/>
     </row>
     <row r="377">
       <c r="C377" s="7" t="n"/>
@@ -5644,6 +6025,7 @@
       <c r="V377" s="7" t="n"/>
       <c r="Y377" s="7" t="n"/>
       <c r="AB377" s="7" t="n"/>
+      <c r="AC377" s="7" t="n"/>
     </row>
     <row r="378">
       <c r="C378" s="7" t="n"/>
@@ -5657,6 +6039,7 @@
       <c r="V378" s="7" t="n"/>
       <c r="Y378" s="7" t="n"/>
       <c r="AB378" s="7" t="n"/>
+      <c r="AC378" s="7" t="n"/>
     </row>
     <row r="379">
       <c r="C379" s="7" t="n"/>
@@ -5670,6 +6053,7 @@
       <c r="V379" s="7" t="n"/>
       <c r="Y379" s="7" t="n"/>
       <c r="AB379" s="7" t="n"/>
+      <c r="AC379" s="7" t="n"/>
     </row>
     <row r="380">
       <c r="C380" s="7" t="n"/>
@@ -5683,6 +6067,7 @@
       <c r="V380" s="7" t="n"/>
       <c r="Y380" s="7" t="n"/>
       <c r="AB380" s="7" t="n"/>
+      <c r="AC380" s="7" t="n"/>
     </row>
     <row r="381">
       <c r="C381" s="7" t="n"/>
@@ -5696,6 +6081,7 @@
       <c r="V381" s="7" t="n"/>
       <c r="Y381" s="7" t="n"/>
       <c r="AB381" s="7" t="n"/>
+      <c r="AC381" s="7" t="n"/>
     </row>
     <row r="382">
       <c r="C382" s="7" t="n"/>
@@ -5709,6 +6095,7 @@
       <c r="V382" s="7" t="n"/>
       <c r="Y382" s="7" t="n"/>
       <c r="AB382" s="7" t="n"/>
+      <c r="AC382" s="7" t="n"/>
     </row>
     <row r="383">
       <c r="C383" s="7" t="n"/>
@@ -5722,6 +6109,7 @@
       <c r="V383" s="7" t="n"/>
       <c r="Y383" s="7" t="n"/>
       <c r="AB383" s="7" t="n"/>
+      <c r="AC383" s="7" t="n"/>
     </row>
     <row r="384">
       <c r="C384" s="7" t="n"/>
@@ -5735,6 +6123,7 @@
       <c r="V384" s="7" t="n"/>
       <c r="Y384" s="7" t="n"/>
       <c r="AB384" s="7" t="n"/>
+      <c r="AC384" s="7" t="n"/>
     </row>
     <row r="385">
       <c r="C385" s="7" t="n"/>
@@ -5748,6 +6137,7 @@
       <c r="V385" s="7" t="n"/>
       <c r="Y385" s="7" t="n"/>
       <c r="AB385" s="7" t="n"/>
+      <c r="AC385" s="7" t="n"/>
     </row>
     <row r="386">
       <c r="C386" s="7" t="n"/>
@@ -5761,6 +6151,7 @@
       <c r="V386" s="7" t="n"/>
       <c r="Y386" s="7" t="n"/>
       <c r="AB386" s="7" t="n"/>
+      <c r="AC386" s="7" t="n"/>
     </row>
     <row r="387">
       <c r="C387" s="7" t="n"/>
@@ -5774,6 +6165,7 @@
       <c r="V387" s="7" t="n"/>
       <c r="Y387" s="7" t="n"/>
       <c r="AB387" s="7" t="n"/>
+      <c r="AC387" s="7" t="n"/>
     </row>
     <row r="388">
       <c r="C388" s="7" t="n"/>
@@ -5787,6 +6179,7 @@
       <c r="V388" s="7" t="n"/>
       <c r="Y388" s="7" t="n"/>
       <c r="AB388" s="7" t="n"/>
+      <c r="AC388" s="7" t="n"/>
     </row>
     <row r="389">
       <c r="C389" s="7" t="n"/>
@@ -5800,6 +6193,7 @@
       <c r="V389" s="7" t="n"/>
       <c r="Y389" s="7" t="n"/>
       <c r="AB389" s="7" t="n"/>
+      <c r="AC389" s="7" t="n"/>
     </row>
     <row r="390">
       <c r="C390" s="7" t="n"/>
@@ -5813,6 +6207,7 @@
       <c r="V390" s="7" t="n"/>
       <c r="Y390" s="7" t="n"/>
       <c r="AB390" s="7" t="n"/>
+      <c r="AC390" s="7" t="n"/>
     </row>
     <row r="391">
       <c r="C391" s="7" t="n"/>
@@ -5826,6 +6221,7 @@
       <c r="V391" s="7" t="n"/>
       <c r="Y391" s="7" t="n"/>
       <c r="AB391" s="7" t="n"/>
+      <c r="AC391" s="7" t="n"/>
     </row>
     <row r="392">
       <c r="C392" s="7" t="n"/>
@@ -5839,6 +6235,7 @@
       <c r="V392" s="7" t="n"/>
       <c r="Y392" s="7" t="n"/>
       <c r="AB392" s="7" t="n"/>
+      <c r="AC392" s="7" t="n"/>
     </row>
     <row r="393">
       <c r="C393" s="7" t="n"/>
@@ -5852,6 +6249,7 @@
       <c r="V393" s="7" t="n"/>
       <c r="Y393" s="7" t="n"/>
       <c r="AB393" s="7" t="n"/>
+      <c r="AC393" s="7" t="n"/>
     </row>
     <row r="394">
       <c r="C394" s="7" t="n"/>
@@ -5865,6 +6263,7 @@
       <c r="V394" s="7" t="n"/>
       <c r="Y394" s="7" t="n"/>
       <c r="AB394" s="7" t="n"/>
+      <c r="AC394" s="7" t="n"/>
     </row>
     <row r="395">
       <c r="C395" s="7" t="n"/>
@@ -5878,6 +6277,7 @@
       <c r="V395" s="7" t="n"/>
       <c r="Y395" s="7" t="n"/>
       <c r="AB395" s="7" t="n"/>
+      <c r="AC395" s="7" t="n"/>
     </row>
     <row r="396">
       <c r="C396" s="7" t="n"/>
@@ -5891,6 +6291,7 @@
       <c r="V396" s="7" t="n"/>
       <c r="Y396" s="7" t="n"/>
       <c r="AB396" s="7" t="n"/>
+      <c r="AC396" s="7" t="n"/>
     </row>
     <row r="397">
       <c r="C397" s="7" t="n"/>
@@ -5904,6 +6305,7 @@
       <c r="V397" s="7" t="n"/>
       <c r="Y397" s="7" t="n"/>
       <c r="AB397" s="7" t="n"/>
+      <c r="AC397" s="7" t="n"/>
     </row>
     <row r="398">
       <c r="C398" s="7" t="n"/>
@@ -5917,6 +6319,7 @@
       <c r="V398" s="7" t="n"/>
       <c r="Y398" s="7" t="n"/>
       <c r="AB398" s="7" t="n"/>
+      <c r="AC398" s="7" t="n"/>
     </row>
     <row r="399">
       <c r="C399" s="7" t="n"/>
@@ -5930,6 +6333,7 @@
       <c r="V399" s="7" t="n"/>
       <c r="Y399" s="7" t="n"/>
       <c r="AB399" s="7" t="n"/>
+      <c r="AC399" s="7" t="n"/>
     </row>
     <row r="400">
       <c r="C400" s="7" t="n"/>
@@ -5943,6 +6347,7 @@
       <c r="V400" s="7" t="n"/>
       <c r="Y400" s="7" t="n"/>
       <c r="AB400" s="7" t="n"/>
+      <c r="AC400" s="7" t="n"/>
     </row>
     <row r="401">
       <c r="C401" s="7" t="n"/>
@@ -5956,6 +6361,7 @@
       <c r="V401" s="7" t="n"/>
       <c r="Y401" s="7" t="n"/>
       <c r="AB401" s="7" t="n"/>
+      <c r="AC401" s="7" t="n"/>
     </row>
     <row r="402">
       <c r="C402" s="7" t="n"/>
@@ -5969,6 +6375,7 @@
       <c r="V402" s="7" t="n"/>
       <c r="Y402" s="7" t="n"/>
       <c r="AB402" s="7" t="n"/>
+      <c r="AC402" s="7" t="n"/>
     </row>
     <row r="403">
       <c r="C403" s="7" t="n"/>
@@ -5982,6 +6389,7 @@
       <c r="V403" s="7" t="n"/>
       <c r="Y403" s="7" t="n"/>
       <c r="AB403" s="7" t="n"/>
+      <c r="AC403" s="7" t="n"/>
     </row>
     <row r="404">
       <c r="C404" s="7" t="n"/>
@@ -5995,6 +6403,7 @@
       <c r="V404" s="7" t="n"/>
       <c r="Y404" s="7" t="n"/>
       <c r="AB404" s="7" t="n"/>
+      <c r="AC404" s="7" t="n"/>
     </row>
     <row r="405">
       <c r="C405" s="7" t="n"/>
@@ -6008,6 +6417,7 @@
       <c r="V405" s="7" t="n"/>
       <c r="Y405" s="7" t="n"/>
       <c r="AB405" s="7" t="n"/>
+      <c r="AC405" s="7" t="n"/>
     </row>
     <row r="406">
       <c r="C406" s="7" t="n"/>
@@ -6021,6 +6431,7 @@
       <c r="V406" s="7" t="n"/>
       <c r="Y406" s="7" t="n"/>
       <c r="AB406" s="7" t="n"/>
+      <c r="AC406" s="7" t="n"/>
     </row>
     <row r="407">
       <c r="C407" s="7" t="n"/>
@@ -6034,6 +6445,7 @@
       <c r="V407" s="7" t="n"/>
       <c r="Y407" s="7" t="n"/>
       <c r="AB407" s="7" t="n"/>
+      <c r="AC407" s="7" t="n"/>
     </row>
     <row r="408">
       <c r="C408" s="7" t="n"/>
@@ -6047,6 +6459,7 @@
       <c r="V408" s="7" t="n"/>
       <c r="Y408" s="7" t="n"/>
       <c r="AB408" s="7" t="n"/>
+      <c r="AC408" s="7" t="n"/>
     </row>
     <row r="409">
       <c r="C409" s="7" t="n"/>
@@ -6060,6 +6473,7 @@
       <c r="V409" s="7" t="n"/>
       <c r="Y409" s="7" t="n"/>
       <c r="AB409" s="7" t="n"/>
+      <c r="AC409" s="7" t="n"/>
     </row>
     <row r="410">
       <c r="C410" s="7" t="n"/>
@@ -6073,6 +6487,7 @@
       <c r="V410" s="7" t="n"/>
       <c r="Y410" s="7" t="n"/>
       <c r="AB410" s="7" t="n"/>
+      <c r="AC410" s="7" t="n"/>
     </row>
     <row r="411">
       <c r="C411" s="7" t="n"/>
@@ -6086,6 +6501,7 @@
       <c r="V411" s="7" t="n"/>
       <c r="Y411" s="7" t="n"/>
       <c r="AB411" s="7" t="n"/>
+      <c r="AC411" s="7" t="n"/>
     </row>
     <row r="412">
       <c r="C412" s="7" t="n"/>
@@ -6099,6 +6515,7 @@
       <c r="V412" s="7" t="n"/>
       <c r="Y412" s="7" t="n"/>
       <c r="AB412" s="7" t="n"/>
+      <c r="AC412" s="7" t="n"/>
     </row>
     <row r="413">
       <c r="C413" s="7" t="n"/>
@@ -6112,6 +6529,7 @@
       <c r="V413" s="7" t="n"/>
       <c r="Y413" s="7" t="n"/>
       <c r="AB413" s="7" t="n"/>
+      <c r="AC413" s="7" t="n"/>
     </row>
     <row r="414">
       <c r="C414" s="7" t="n"/>
@@ -6125,6 +6543,7 @@
       <c r="V414" s="7" t="n"/>
       <c r="Y414" s="7" t="n"/>
       <c r="AB414" s="7" t="n"/>
+      <c r="AC414" s="7" t="n"/>
     </row>
     <row r="415">
       <c r="C415" s="7" t="n"/>
@@ -6138,6 +6557,7 @@
       <c r="V415" s="7" t="n"/>
       <c r="Y415" s="7" t="n"/>
       <c r="AB415" s="7" t="n"/>
+      <c r="AC415" s="7" t="n"/>
     </row>
     <row r="416">
       <c r="C416" s="7" t="n"/>
@@ -6151,6 +6571,7 @@
       <c r="V416" s="7" t="n"/>
       <c r="Y416" s="7" t="n"/>
       <c r="AB416" s="7" t="n"/>
+      <c r="AC416" s="7" t="n"/>
     </row>
     <row r="417">
       <c r="C417" s="7" t="n"/>
@@ -6164,6 +6585,7 @@
       <c r="V417" s="7" t="n"/>
       <c r="Y417" s="7" t="n"/>
       <c r="AB417" s="7" t="n"/>
+      <c r="AC417" s="7" t="n"/>
     </row>
     <row r="418">
       <c r="C418" s="7" t="n"/>
@@ -6177,6 +6599,7 @@
       <c r="V418" s="7" t="n"/>
       <c r="Y418" s="7" t="n"/>
       <c r="AB418" s="7" t="n"/>
+      <c r="AC418" s="7" t="n"/>
     </row>
     <row r="419">
       <c r="C419" s="7" t="n"/>
@@ -6190,6 +6613,7 @@
       <c r="V419" s="7" t="n"/>
       <c r="Y419" s="7" t="n"/>
       <c r="AB419" s="7" t="n"/>
+      <c r="AC419" s="7" t="n"/>
     </row>
     <row r="420">
       <c r="C420" s="7" t="n"/>
@@ -6203,6 +6627,7 @@
       <c r="V420" s="7" t="n"/>
       <c r="Y420" s="7" t="n"/>
       <c r="AB420" s="7" t="n"/>
+      <c r="AC420" s="7" t="n"/>
     </row>
     <row r="421">
       <c r="C421" s="7" t="n"/>
@@ -6216,6 +6641,7 @@
       <c r="V421" s="7" t="n"/>
       <c r="Y421" s="7" t="n"/>
       <c r="AB421" s="7" t="n"/>
+      <c r="AC421" s="7" t="n"/>
     </row>
     <row r="422">
       <c r="C422" s="7" t="n"/>
@@ -6229,6 +6655,7 @@
       <c r="V422" s="7" t="n"/>
       <c r="Y422" s="7" t="n"/>
       <c r="AB422" s="7" t="n"/>
+      <c r="AC422" s="7" t="n"/>
     </row>
     <row r="423">
       <c r="C423" s="7" t="n"/>
@@ -6242,6 +6669,7 @@
       <c r="V423" s="7" t="n"/>
       <c r="Y423" s="7" t="n"/>
       <c r="AB423" s="7" t="n"/>
+      <c r="AC423" s="7" t="n"/>
     </row>
     <row r="424">
       <c r="C424" s="7" t="n"/>
@@ -6255,6 +6683,7 @@
       <c r="V424" s="7" t="n"/>
       <c r="Y424" s="7" t="n"/>
       <c r="AB424" s="7" t="n"/>
+      <c r="AC424" s="7" t="n"/>
     </row>
     <row r="425">
       <c r="C425" s="7" t="n"/>
@@ -6268,6 +6697,7 @@
       <c r="V425" s="7" t="n"/>
       <c r="Y425" s="7" t="n"/>
       <c r="AB425" s="7" t="n"/>
+      <c r="AC425" s="7" t="n"/>
     </row>
     <row r="426">
       <c r="C426" s="7" t="n"/>
@@ -6281,6 +6711,7 @@
       <c r="V426" s="7" t="n"/>
       <c r="Y426" s="7" t="n"/>
       <c r="AB426" s="7" t="n"/>
+      <c r="AC426" s="7" t="n"/>
     </row>
     <row r="427">
       <c r="C427" s="7" t="n"/>
@@ -6294,6 +6725,7 @@
       <c r="V427" s="7" t="n"/>
       <c r="Y427" s="7" t="n"/>
       <c r="AB427" s="7" t="n"/>
+      <c r="AC427" s="7" t="n"/>
     </row>
     <row r="428">
       <c r="C428" s="7" t="n"/>
@@ -6307,6 +6739,7 @@
       <c r="V428" s="7" t="n"/>
       <c r="Y428" s="7" t="n"/>
       <c r="AB428" s="7" t="n"/>
+      <c r="AC428" s="7" t="n"/>
     </row>
     <row r="429">
       <c r="C429" s="7" t="n"/>
@@ -6320,6 +6753,7 @@
       <c r="V429" s="7" t="n"/>
       <c r="Y429" s="7" t="n"/>
       <c r="AB429" s="7" t="n"/>
+      <c r="AC429" s="7" t="n"/>
     </row>
     <row r="430">
       <c r="C430" s="7" t="n"/>
@@ -6333,6 +6767,7 @@
       <c r="V430" s="7" t="n"/>
       <c r="Y430" s="7" t="n"/>
       <c r="AB430" s="7" t="n"/>
+      <c r="AC430" s="7" t="n"/>
     </row>
     <row r="431">
       <c r="C431" s="7" t="n"/>
@@ -6346,6 +6781,7 @@
       <c r="V431" s="7" t="n"/>
       <c r="Y431" s="7" t="n"/>
       <c r="AB431" s="7" t="n"/>
+      <c r="AC431" s="7" t="n"/>
     </row>
     <row r="432">
       <c r="C432" s="7" t="n"/>
@@ -6359,6 +6795,7 @@
       <c r="V432" s="7" t="n"/>
       <c r="Y432" s="7" t="n"/>
       <c r="AB432" s="7" t="n"/>
+      <c r="AC432" s="7" t="n"/>
     </row>
     <row r="433">
       <c r="C433" s="7" t="n"/>
@@ -6372,6 +6809,7 @@
       <c r="V433" s="7" t="n"/>
       <c r="Y433" s="7" t="n"/>
       <c r="AB433" s="7" t="n"/>
+      <c r="AC433" s="7" t="n"/>
     </row>
     <row r="434">
       <c r="C434" s="7" t="n"/>
@@ -6385,6 +6823,7 @@
       <c r="V434" s="7" t="n"/>
       <c r="Y434" s="7" t="n"/>
       <c r="AB434" s="7" t="n"/>
+      <c r="AC434" s="7" t="n"/>
     </row>
     <row r="435">
       <c r="C435" s="7" t="n"/>
@@ -6398,6 +6837,7 @@
       <c r="V435" s="7" t="n"/>
       <c r="Y435" s="7" t="n"/>
       <c r="AB435" s="7" t="n"/>
+      <c r="AC435" s="7" t="n"/>
     </row>
     <row r="436">
       <c r="C436" s="7" t="n"/>
@@ -6411,6 +6851,7 @@
       <c r="V436" s="7" t="n"/>
       <c r="Y436" s="7" t="n"/>
       <c r="AB436" s="7" t="n"/>
+      <c r="AC436" s="7" t="n"/>
     </row>
     <row r="437">
       <c r="C437" s="7" t="n"/>
@@ -6424,6 +6865,7 @@
       <c r="V437" s="7" t="n"/>
       <c r="Y437" s="7" t="n"/>
       <c r="AB437" s="7" t="n"/>
+      <c r="AC437" s="7" t="n"/>
     </row>
     <row r="438">
       <c r="C438" s="7" t="n"/>
@@ -6437,6 +6879,7 @@
       <c r="V438" s="7" t="n"/>
       <c r="Y438" s="7" t="n"/>
       <c r="AB438" s="7" t="n"/>
+      <c r="AC438" s="7" t="n"/>
     </row>
     <row r="439">
       <c r="C439" s="7" t="n"/>
@@ -6450,6 +6893,7 @@
       <c r="V439" s="7" t="n"/>
       <c r="Y439" s="7" t="n"/>
       <c r="AB439" s="7" t="n"/>
+      <c r="AC439" s="7" t="n"/>
     </row>
     <row r="440">
       <c r="C440" s="7" t="n"/>
@@ -6463,6 +6907,7 @@
       <c r="V440" s="7" t="n"/>
       <c r="Y440" s="7" t="n"/>
       <c r="AB440" s="7" t="n"/>
+      <c r="AC440" s="7" t="n"/>
     </row>
     <row r="441">
       <c r="C441" s="7" t="n"/>
@@ -6476,6 +6921,7 @@
       <c r="V441" s="7" t="n"/>
       <c r="Y441" s="7" t="n"/>
       <c r="AB441" s="7" t="n"/>
+      <c r="AC441" s="7" t="n"/>
     </row>
     <row r="442">
       <c r="C442" s="7" t="n"/>
@@ -6489,6 +6935,7 @@
       <c r="V442" s="7" t="n"/>
       <c r="Y442" s="7" t="n"/>
       <c r="AB442" s="7" t="n"/>
+      <c r="AC442" s="7" t="n"/>
     </row>
     <row r="443">
       <c r="C443" s="7" t="n"/>
@@ -6502,6 +6949,7 @@
       <c r="V443" s="7" t="n"/>
       <c r="Y443" s="7" t="n"/>
       <c r="AB443" s="7" t="n"/>
+      <c r="AC443" s="7" t="n"/>
     </row>
     <row r="444">
       <c r="C444" s="7" t="n"/>
@@ -6515,6 +6963,7 @@
       <c r="V444" s="7" t="n"/>
       <c r="Y444" s="7" t="n"/>
       <c r="AB444" s="7" t="n"/>
+      <c r="AC444" s="7" t="n"/>
     </row>
     <row r="445">
       <c r="C445" s="7" t="n"/>
@@ -6528,6 +6977,7 @@
       <c r="V445" s="7" t="n"/>
       <c r="Y445" s="7" t="n"/>
       <c r="AB445" s="7" t="n"/>
+      <c r="AC445" s="7" t="n"/>
     </row>
     <row r="446">
       <c r="C446" s="7" t="n"/>
@@ -6541,6 +6991,7 @@
       <c r="V446" s="7" t="n"/>
       <c r="Y446" s="7" t="n"/>
       <c r="AB446" s="7" t="n"/>
+      <c r="AC446" s="7" t="n"/>
     </row>
     <row r="447">
       <c r="C447" s="7" t="n"/>
@@ -6554,6 +7005,7 @@
       <c r="V447" s="7" t="n"/>
       <c r="Y447" s="7" t="n"/>
       <c r="AB447" s="7" t="n"/>
+      <c r="AC447" s="7" t="n"/>
     </row>
     <row r="448">
       <c r="C448" s="7" t="n"/>
@@ -6567,6 +7019,7 @@
       <c r="V448" s="7" t="n"/>
       <c r="Y448" s="7" t="n"/>
       <c r="AB448" s="7" t="n"/>
+      <c r="AC448" s="7" t="n"/>
     </row>
     <row r="449">
       <c r="C449" s="7" t="n"/>
@@ -6580,6 +7033,7 @@
       <c r="V449" s="7" t="n"/>
       <c r="Y449" s="7" t="n"/>
       <c r="AB449" s="7" t="n"/>
+      <c r="AC449" s="7" t="n"/>
     </row>
     <row r="450">
       <c r="C450" s="7" t="n"/>
@@ -6593,6 +7047,7 @@
       <c r="V450" s="7" t="n"/>
       <c r="Y450" s="7" t="n"/>
       <c r="AB450" s="7" t="n"/>
+      <c r="AC450" s="7" t="n"/>
     </row>
     <row r="451">
       <c r="C451" s="7" t="n"/>
@@ -6606,6 +7061,7 @@
       <c r="V451" s="7" t="n"/>
       <c r="Y451" s="7" t="n"/>
       <c r="AB451" s="7" t="n"/>
+      <c r="AC451" s="7" t="n"/>
     </row>
     <row r="452">
       <c r="C452" s="7" t="n"/>
@@ -6619,6 +7075,7 @@
       <c r="V452" s="7" t="n"/>
       <c r="Y452" s="7" t="n"/>
       <c r="AB452" s="7" t="n"/>
+      <c r="AC452" s="7" t="n"/>
     </row>
     <row r="453">
       <c r="C453" s="7" t="n"/>
@@ -6632,6 +7089,7 @@
       <c r="V453" s="7" t="n"/>
       <c r="Y453" s="7" t="n"/>
       <c r="AB453" s="7" t="n"/>
+      <c r="AC453" s="7" t="n"/>
     </row>
     <row r="454">
       <c r="C454" s="7" t="n"/>
@@ -6645,6 +7103,7 @@
       <c r="V454" s="7" t="n"/>
       <c r="Y454" s="7" t="n"/>
       <c r="AB454" s="7" t="n"/>
+      <c r="AC454" s="7" t="n"/>
     </row>
     <row r="455">
       <c r="C455" s="7" t="n"/>
@@ -6658,6 +7117,7 @@
       <c r="V455" s="7" t="n"/>
       <c r="Y455" s="7" t="n"/>
       <c r="AB455" s="7" t="n"/>
+      <c r="AC455" s="7" t="n"/>
     </row>
     <row r="456">
       <c r="C456" s="7" t="n"/>
@@ -6671,6 +7131,7 @@
       <c r="V456" s="7" t="n"/>
       <c r="Y456" s="7" t="n"/>
       <c r="AB456" s="7" t="n"/>
+      <c r="AC456" s="7" t="n"/>
     </row>
     <row r="457">
       <c r="C457" s="7" t="n"/>
@@ -6684,6 +7145,7 @@
       <c r="V457" s="7" t="n"/>
       <c r="Y457" s="7" t="n"/>
       <c r="AB457" s="7" t="n"/>
+      <c r="AC457" s="7" t="n"/>
     </row>
     <row r="458">
       <c r="C458" s="7" t="n"/>
@@ -6697,6 +7159,7 @@
       <c r="V458" s="7" t="n"/>
       <c r="Y458" s="7" t="n"/>
       <c r="AB458" s="7" t="n"/>
+      <c r="AC458" s="7" t="n"/>
     </row>
     <row r="459">
       <c r="C459" s="7" t="n"/>
@@ -6710,6 +7173,7 @@
       <c r="V459" s="7" t="n"/>
       <c r="Y459" s="7" t="n"/>
       <c r="AB459" s="7" t="n"/>
+      <c r="AC459" s="7" t="n"/>
     </row>
     <row r="460">
       <c r="C460" s="7" t="n"/>
@@ -6723,6 +7187,7 @@
       <c r="V460" s="7" t="n"/>
       <c r="Y460" s="7" t="n"/>
       <c r="AB460" s="7" t="n"/>
+      <c r="AC460" s="7" t="n"/>
     </row>
     <row r="461">
       <c r="C461" s="7" t="n"/>
@@ -6736,6 +7201,7 @@
       <c r="V461" s="7" t="n"/>
       <c r="Y461" s="7" t="n"/>
       <c r="AB461" s="7" t="n"/>
+      <c r="AC461" s="7" t="n"/>
     </row>
     <row r="462">
       <c r="C462" s="7" t="n"/>
@@ -6749,6 +7215,7 @@
       <c r="V462" s="7" t="n"/>
       <c r="Y462" s="7" t="n"/>
       <c r="AB462" s="7" t="n"/>
+      <c r="AC462" s="7" t="n"/>
     </row>
     <row r="463">
       <c r="C463" s="7" t="n"/>
@@ -6762,6 +7229,7 @@
       <c r="V463" s="7" t="n"/>
       <c r="Y463" s="7" t="n"/>
       <c r="AB463" s="7" t="n"/>
+      <c r="AC463" s="7" t="n"/>
     </row>
     <row r="464">
       <c r="C464" s="7" t="n"/>
@@ -6775,6 +7243,7 @@
       <c r="V464" s="7" t="n"/>
       <c r="Y464" s="7" t="n"/>
       <c r="AB464" s="7" t="n"/>
+      <c r="AC464" s="7" t="n"/>
     </row>
     <row r="465">
       <c r="C465" s="7" t="n"/>
@@ -6788,6 +7257,7 @@
       <c r="V465" s="7" t="n"/>
       <c r="Y465" s="7" t="n"/>
       <c r="AB465" s="7" t="n"/>
+      <c r="AC465" s="7" t="n"/>
     </row>
     <row r="466">
       <c r="C466" s="7" t="n"/>
@@ -6801,6 +7271,7 @@
       <c r="V466" s="7" t="n"/>
       <c r="Y466" s="7" t="n"/>
       <c r="AB466" s="7" t="n"/>
+      <c r="AC466" s="7" t="n"/>
     </row>
     <row r="467">
       <c r="C467" s="7" t="n"/>
@@ -6814,6 +7285,7 @@
       <c r="V467" s="7" t="n"/>
       <c r="Y467" s="7" t="n"/>
       <c r="AB467" s="7" t="n"/>
+      <c r="AC467" s="7" t="n"/>
     </row>
     <row r="468">
       <c r="C468" s="7" t="n"/>
@@ -6827,6 +7299,7 @@
       <c r="V468" s="7" t="n"/>
       <c r="Y468" s="7" t="n"/>
       <c r="AB468" s="7" t="n"/>
+      <c r="AC468" s="7" t="n"/>
     </row>
     <row r="469">
       <c r="C469" s="7" t="n"/>
@@ -6840,6 +7313,7 @@
       <c r="V469" s="7" t="n"/>
       <c r="Y469" s="7" t="n"/>
       <c r="AB469" s="7" t="n"/>
+      <c r="AC469" s="7" t="n"/>
     </row>
     <row r="470">
       <c r="C470" s="7" t="n"/>
@@ -6853,6 +7327,7 @@
       <c r="V470" s="7" t="n"/>
       <c r="Y470" s="7" t="n"/>
       <c r="AB470" s="7" t="n"/>
+      <c r="AC470" s="7" t="n"/>
     </row>
     <row r="471">
       <c r="C471" s="7" t="n"/>
@@ -6866,6 +7341,7 @@
       <c r="V471" s="7" t="n"/>
       <c r="Y471" s="7" t="n"/>
       <c r="AB471" s="7" t="n"/>
+      <c r="AC471" s="7" t="n"/>
     </row>
     <row r="472">
       <c r="C472" s="7" t="n"/>
@@ -6879,6 +7355,7 @@
       <c r="V472" s="7" t="n"/>
       <c r="Y472" s="7" t="n"/>
       <c r="AB472" s="7" t="n"/>
+      <c r="AC472" s="7" t="n"/>
     </row>
     <row r="473">
       <c r="C473" s="7" t="n"/>
@@ -6892,6 +7369,7 @@
       <c r="V473" s="7" t="n"/>
       <c r="Y473" s="7" t="n"/>
       <c r="AB473" s="7" t="n"/>
+      <c r="AC473" s="7" t="n"/>
     </row>
     <row r="474">
       <c r="C474" s="7" t="n"/>
@@ -6905,6 +7383,7 @@
       <c r="V474" s="7" t="n"/>
       <c r="Y474" s="7" t="n"/>
       <c r="AB474" s="7" t="n"/>
+      <c r="AC474" s="7" t="n"/>
     </row>
     <row r="475">
       <c r="C475" s="7" t="n"/>
@@ -6918,6 +7397,7 @@
       <c r="V475" s="7" t="n"/>
       <c r="Y475" s="7" t="n"/>
       <c r="AB475" s="7" t="n"/>
+      <c r="AC475" s="7" t="n"/>
     </row>
     <row r="476">
       <c r="C476" s="7" t="n"/>
@@ -6931,6 +7411,7 @@
       <c r="V476" s="7" t="n"/>
       <c r="Y476" s="7" t="n"/>
       <c r="AB476" s="7" t="n"/>
+      <c r="AC476" s="7" t="n"/>
     </row>
     <row r="477">
       <c r="C477" s="7" t="n"/>
@@ -6944,6 +7425,7 @@
       <c r="V477" s="7" t="n"/>
       <c r="Y477" s="7" t="n"/>
       <c r="AB477" s="7" t="n"/>
+      <c r="AC477" s="7" t="n"/>
     </row>
     <row r="478">
       <c r="C478" s="7" t="n"/>
@@ -6957,6 +7439,7 @@
       <c r="V478" s="7" t="n"/>
       <c r="Y478" s="7" t="n"/>
       <c r="AB478" s="7" t="n"/>
+      <c r="AC478" s="7" t="n"/>
     </row>
     <row r="479">
       <c r="C479" s="7" t="n"/>
@@ -6970,6 +7453,7 @@
       <c r="V479" s="7" t="n"/>
       <c r="Y479" s="7" t="n"/>
       <c r="AB479" s="7" t="n"/>
+      <c r="AC479" s="7" t="n"/>
     </row>
     <row r="480">
       <c r="C480" s="7" t="n"/>
@@ -6983,6 +7467,7 @@
       <c r="V480" s="7" t="n"/>
       <c r="Y480" s="7" t="n"/>
       <c r="AB480" s="7" t="n"/>
+      <c r="AC480" s="7" t="n"/>
     </row>
     <row r="481">
       <c r="C481" s="7" t="n"/>
@@ -6996,6 +7481,7 @@
       <c r="V481" s="7" t="n"/>
       <c r="Y481" s="7" t="n"/>
       <c r="AB481" s="7" t="n"/>
+      <c r="AC481" s="7" t="n"/>
     </row>
     <row r="482">
       <c r="C482" s="7" t="n"/>
@@ -7009,6 +7495,7 @@
       <c r="V482" s="7" t="n"/>
       <c r="Y482" s="7" t="n"/>
       <c r="AB482" s="7" t="n"/>
+      <c r="AC482" s="7" t="n"/>
     </row>
     <row r="483">
       <c r="C483" s="7" t="n"/>
@@ -7022,6 +7509,7 @@
       <c r="V483" s="7" t="n"/>
       <c r="Y483" s="7" t="n"/>
       <c r="AB483" s="7" t="n"/>
+      <c r="AC483" s="7" t="n"/>
     </row>
     <row r="484">
       <c r="C484" s="7" t="n"/>
@@ -7035,6 +7523,7 @@
       <c r="V484" s="7" t="n"/>
       <c r="Y484" s="7" t="n"/>
       <c r="AB484" s="7" t="n"/>
+      <c r="AC484" s="7" t="n"/>
     </row>
     <row r="485">
       <c r="C485" s="7" t="n"/>
@@ -7048,6 +7537,7 @@
       <c r="V485" s="7" t="n"/>
       <c r="Y485" s="7" t="n"/>
       <c r="AB485" s="7" t="n"/>
+      <c r="AC485" s="7" t="n"/>
     </row>
     <row r="486">
       <c r="C486" s="7" t="n"/>
@@ -7061,6 +7551,7 @@
       <c r="V486" s="7" t="n"/>
       <c r="Y486" s="7" t="n"/>
       <c r="AB486" s="7" t="n"/>
+      <c r="AC486" s="7" t="n"/>
     </row>
     <row r="487">
       <c r="C487" s="7" t="n"/>
@@ -7074,6 +7565,7 @@
       <c r="V487" s="7" t="n"/>
       <c r="Y487" s="7" t="n"/>
       <c r="AB487" s="7" t="n"/>
+      <c r="AC487" s="7" t="n"/>
     </row>
     <row r="488">
       <c r="C488" s="7" t="n"/>
@@ -7087,6 +7579,7 @@
       <c r="V488" s="7" t="n"/>
       <c r="Y488" s="7" t="n"/>
       <c r="AB488" s="7" t="n"/>
+      <c r="AC488" s="7" t="n"/>
     </row>
     <row r="489">
       <c r="C489" s="7" t="n"/>
@@ -7100,6 +7593,7 @@
       <c r="V489" s="7" t="n"/>
       <c r="Y489" s="7" t="n"/>
       <c r="AB489" s="7" t="n"/>
+      <c r="AC489" s="7" t="n"/>
     </row>
     <row r="490">
       <c r="C490" s="7" t="n"/>
@@ -7113,6 +7607,7 @@
       <c r="V490" s="7" t="n"/>
       <c r="Y490" s="7" t="n"/>
       <c r="AB490" s="7" t="n"/>
+      <c r="AC490" s="7" t="n"/>
     </row>
     <row r="491">
       <c r="C491" s="7" t="n"/>
@@ -7126,6 +7621,7 @@
       <c r="V491" s="7" t="n"/>
       <c r="Y491" s="7" t="n"/>
       <c r="AB491" s="7" t="n"/>
+      <c r="AC491" s="7" t="n"/>
     </row>
     <row r="492">
       <c r="C492" s="7" t="n"/>
@@ -7139,6 +7635,7 @@
       <c r="V492" s="7" t="n"/>
       <c r="Y492" s="7" t="n"/>
       <c r="AB492" s="7" t="n"/>
+      <c r="AC492" s="7" t="n"/>
     </row>
     <row r="493">
       <c r="C493" s="7" t="n"/>
@@ -7152,6 +7649,7 @@
       <c r="V493" s="7" t="n"/>
       <c r="Y493" s="7" t="n"/>
       <c r="AB493" s="7" t="n"/>
+      <c r="AC493" s="7" t="n"/>
     </row>
     <row r="494">
       <c r="C494" s="7" t="n"/>
@@ -7165,6 +7663,7 @@
       <c r="V494" s="7" t="n"/>
       <c r="Y494" s="7" t="n"/>
       <c r="AB494" s="7" t="n"/>
+      <c r="AC494" s="7" t="n"/>
     </row>
     <row r="495">
       <c r="C495" s="7" t="n"/>
@@ -7178,6 +7677,7 @@
       <c r="V495" s="7" t="n"/>
       <c r="Y495" s="7" t="n"/>
       <c r="AB495" s="7" t="n"/>
+      <c r="AC495" s="7" t="n"/>
     </row>
     <row r="496">
       <c r="C496" s="7" t="n"/>
@@ -7191,6 +7691,7 @@
       <c r="V496" s="7" t="n"/>
       <c r="Y496" s="7" t="n"/>
       <c r="AB496" s="7" t="n"/>
+      <c r="AC496" s="7" t="n"/>
     </row>
     <row r="497">
       <c r="C497" s="7" t="n"/>
@@ -7204,6 +7705,7 @@
       <c r="V497" s="7" t="n"/>
       <c r="Y497" s="7" t="n"/>
       <c r="AB497" s="7" t="n"/>
+      <c r="AC497" s="7" t="n"/>
     </row>
     <row r="498">
       <c r="C498" s="7" t="n"/>
@@ -7217,6 +7719,7 @@
       <c r="V498" s="7" t="n"/>
       <c r="Y498" s="7" t="n"/>
       <c r="AB498" s="7" t="n"/>
+      <c r="AC498" s="7" t="n"/>
     </row>
     <row r="499">
       <c r="C499" s="7" t="n"/>
@@ -7230,6 +7733,7 @@
       <c r="V499" s="7" t="n"/>
       <c r="Y499" s="7" t="n"/>
       <c r="AB499" s="7" t="n"/>
+      <c r="AC499" s="7" t="n"/>
     </row>
     <row r="500">
       <c r="C500" s="7" t="n"/>
@@ -7243,6 +7747,7 @@
       <c r="V500" s="7" t="n"/>
       <c r="Y500" s="7" t="n"/>
       <c r="AB500" s="7" t="n"/>
+      <c r="AC500" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7255,7 +7760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -7362,6 +7867,13 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Grade: only for classes that have grades (for example Aftercare with Gr R to Gr 12). Type it as Gr 3, Grade 3 or just 3. Leave it blank for any other class.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>